<commit_message>
Dashboard spec: support Excel/CSV upload alongside the WatchOps API
WatchOps API stays the default source for inventory and sales, but Excel/CSV
upload is now also supported — for businesses not on WatchOps, history older than
the API holds, or manual data. New DATA-05 captures the flexible column-mapping
importer (detect columns, user confirms the mapping), which the POC already has.
Updated DATA-01/02 to name both sources and softened the Backlog note.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WatchBI_Dashboard_Requirements.xlsx
+++ b/WatchBI_Dashboard_Requirements.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog &amp; Open Items" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requirements'!$A$1:$J$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requirements'!$A$1:$J$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -231,10 +231,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -747,7 +747,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Inventory AND sales history both come from the WatchOps API (sold items carry price/cost/condition/date). No Excel upload.</t>
+          <t>Inventory and sales history come from the WatchOps API by default. Excel/CSV upload is ALSO supported — for businesses not on WatchOps, history older than the API holds, or manual data — with flexible column mapping.</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Read the business's live inventory from the WatchOps API: cost, target prices, condition, status, inventory type, supplier, serial, payment status, purchase date.</t>
+          <t>Read the business's live inventory from the WatchOps API (default): cost, target prices, condition, status, inventory type, supplier, serial, payment status, purchase date; OR from an uploaded inventory sheet (see DATA-05).</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>Inventory analytics reflect current WatchOps holdings.</t>
+          <t>Inventory analytics reflect current WatchOps holdings, or the uploaded sheet.</t>
         </is>
       </c>
       <c r="J7" s="15" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Read sales history from the WatchOps API: sold items with sold price, cost, condition, salesperson, and dates.</t>
+          <t>Read sales history from the WatchOps API (default): sold items with sold price, cost, condition, salesperson, and dates; OR from an uploaded sales sheet (see DATA-05).</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1243,12 +1243,12 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Sales analytics reflect WatchOps sales; no upload needed.</t>
+          <t>Sales analytics reflect WatchOps sales, or the uploaded sheet.</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>Same source Deal Radar uses. Replaces the POC's Excel upload.</t>
+          <t>API is the default; Excel upload also supported.</t>
         </is>
       </c>
     </row>
@@ -1355,22 +1355,22 @@
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>INV-01</t>
+          <t>DATA-05</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>Inventory Analytics</t>
+          <t>Data Sources</t>
         </is>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>Inventory KPI header: items in stock, capital tied up, count aged 91+ days, median days to sell, overall health.</t>
+          <t>Support uploading inventory and/or sales history via Excel/CSV, as an alternative or supplement to the WatchOps API. The importer shall detect the sheet's columns and let the user confirm the field mapping, so it works with any dealer's export format.</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Admin tier</t>
         </is>
       </c>
       <c r="E11" s="16" t="inlineStr">
@@ -1388,26 +1388,22 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="H11" s="15" t="inlineStr">
-        <is>
-          <t>DATA-01</t>
-        </is>
-      </c>
+      <c r="H11" s="15" t="inlineStr"/>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>Header figures match the underlying inventory.</t>
+          <t>A user uploads a sheet, confirms the column mapping, and the analytics populate from it.</t>
         </is>
       </c>
       <c r="J11" s="15" t="inlineStr">
         <is>
-          <t>Validated in POC.</t>
+          <t>Validated in POC (mapping screen). Covers non-WatchOps businesses and older history.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>INV-02</t>
+          <t>INV-01</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -1417,7 +1413,7 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Inventory breakdowns: by brand, by brand &amp; condition (new/used), by inventory type (owned/memo/partnership/consignment), by price tier, by product line, and by model number.</t>
+          <t>Inventory KPI header: items in stock, capital tied up, count aged 91+ days, median days to sell, overall health.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1442,12 +1438,12 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>DATA-01,DATA-04</t>
+          <t>DATA-01</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Each breakdown totals to the inventory.</t>
+          <t>Header figures match the underlying inventory.</t>
         </is>
       </c>
       <c r="J12" s="11" t="inlineStr">
@@ -1459,7 +1455,7 @@
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>INV-03</t>
+          <t>INV-02</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
@@ -1469,7 +1465,7 @@
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>Inventory aging: age buckets and an A→F quality grade (A = fresh, F = aged) based on days in stock.</t>
+          <t>Inventory breakdowns: by brand, by brand &amp; condition (new/used), by inventory type (owned/memo/partnership/consignment), by price tier, by product line, and by model number.</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
@@ -1494,24 +1490,24 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>DATA-01</t>
+          <t>DATA-01,DATA-04</t>
         </is>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>Each item lands in the correct age bucket / grade.</t>
+          <t>Each breakdown totals to the inventory.</t>
         </is>
       </c>
       <c r="J13" s="15" t="inlineStr">
         <is>
-          <t>Grade thresholds configurable (GRADE-02). Formula in Impl. Notes.</t>
+          <t>Validated in POC.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>INV-04</t>
+          <t>INV-03</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -1521,7 +1517,7 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Sell-through velocity: weekly velocity and weeks-of-stock per model and brand, from recent sales.</t>
+          <t>Inventory aging: age buckets and an A→F quality grade (A = fresh, F = aged) based on days in stock.</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1546,24 +1542,24 @@
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>DATA-01,DATA-02</t>
+          <t>DATA-01</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>Velocity and weeks-of-stock compute per model/brand.</t>
+          <t>Each item lands in the correct age bucket / grade.</t>
         </is>
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
-          <t>Sparse windows must not overstate velocity — see Impl. Notes.</t>
+          <t>Grade thresholds configurable (GRADE-02). Formula in Impl. Notes.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>INV-05</t>
+          <t>INV-04</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
@@ -1573,7 +1569,7 @@
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>Supplier view: spend, units, and aging by supplier (top suppliers).</t>
+          <t>Sell-through velocity: weekly velocity and weeks-of-stock per model and brand, from recent sales.</t>
         </is>
       </c>
       <c r="D15" s="15" t="inlineStr">
@@ -1581,9 +1577,9 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>Should</t>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="F15" s="17" t="inlineStr">
@@ -1598,24 +1594,24 @@
       </c>
       <c r="H15" s="15" t="inlineStr">
         <is>
-          <t>DATA-01</t>
+          <t>DATA-01,DATA-02</t>
         </is>
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>Supplier totals reconcile to inventory.</t>
+          <t>Velocity and weeks-of-stock compute per model/brand.</t>
         </is>
       </c>
       <c r="J15" s="15" t="inlineStr">
         <is>
-          <t>Validated in POC.</t>
+          <t>Sparse windows must not overstate velocity — see Impl. Notes.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>INV-06</t>
+          <t>INV-05</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -1625,7 +1621,7 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Data-quality view: flag inventory with missing/blank key fields (no brand and no model, missing cost, etc.).</t>
+          <t>Supplier view: spend, units, and aging by supplier (top suppliers).</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1633,14 +1629,14 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E16" s="19" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G16" s="13" t="inlineStr">
@@ -1655,19 +1651,19 @@
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>Rows with missing fields are listed and counted.</t>
+          <t>Supplier totals reconcile to inventory.</t>
         </is>
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
-          <t>Fully-blank rows filtered at source dashboard-wide.</t>
+          <t>Validated in POC.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>INV-07</t>
+          <t>INV-06</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
@@ -1677,7 +1673,7 @@
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>Drill-down navigation: brand → product line → model.</t>
+          <t>Data-quality view: flag inventory with missing/blank key fields (no brand and no model, missing cost, etc.).</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
@@ -1685,14 +1681,14 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E17" s="18" t="inlineStr">
+      <c r="E17" s="19" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G17" s="17" t="inlineStr">
@@ -1702,34 +1698,34 @@
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>INV-02</t>
+          <t>DATA-01</t>
         </is>
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>Clicking a brand narrows to its lines and models.</t>
+          <t>Rows with missing fields are listed and counted.</t>
         </is>
       </c>
       <c r="J17" s="15" t="inlineStr">
         <is>
-          <t>Validated in POC.</t>
+          <t>Fully-blank rows filtered at source dashboard-wide.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>SALES-01</t>
+          <t>INV-07</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Sales Analytics</t>
+          <t>Inventory Analytics</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Sales KPI header: revenue, units sold, total profit $, median margin %.</t>
+          <t>Drill-down navigation: brand → product line → model.</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1737,9 +1733,9 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>Must</t>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Should</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr">
@@ -1754,12 +1750,12 @@
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>DATA-02</t>
+          <t>INV-02</t>
         </is>
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>Header figures match the sales set.</t>
+          <t>Clicking a brand narrows to its lines and models.</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr">
@@ -1771,7 +1767,7 @@
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>SALES-02</t>
+          <t>SALES-01</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
@@ -1781,7 +1777,7 @@
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>Salesperson performance: profit, units, and velocity (median days to sell) per salesperson, with drill-down into each sale.</t>
+          <t>Sales KPI header: revenue, units sold, total profit $, median margin %.</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
@@ -1811,19 +1807,19 @@
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
-          <t>Each salesperson's totals reconcile; sales are drillable.</t>
+          <t>Header figures match the sales set.</t>
         </is>
       </c>
       <c r="J19" s="15" t="inlineStr">
         <is>
-          <t>'Everyone sees everyone' per PLAT-05.</t>
+          <t>Validated in POC.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>SALES-03</t>
+          <t>SALES-02</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -1833,7 +1829,7 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Per-sale performance grade (the DJ grade): a points system over margin and velocity (days on hand), grade A–D.</t>
+          <t>Salesperson performance: profit, units, and velocity (median days to sell) per salesperson, with drill-down into each sale.</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -1858,24 +1854,24 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>DATA-02,GRADE-01</t>
+          <t>DATA-02</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>Each sale receives a grade from its margin and days-on-hand.</t>
+          <t>Each salesperson's totals reconcile; sales are drillable.</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
-          <t>Exact formula in Impl. Notes. Does NOT use market data.</t>
+          <t>'Everyone sees everyone' per PLAT-05.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>SALES-04</t>
+          <t>SALES-03</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
@@ -1885,7 +1881,7 @@
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>Sales breakdown by brand &amp; condition: units, revenue, profit, margin.</t>
+          <t>Per-sale performance grade (the DJ grade): a points system over margin and velocity (days on hand), grade A–D.</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
@@ -1893,9 +1889,9 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Should</t>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="F21" s="17" t="inlineStr">
@@ -1910,34 +1906,34 @@
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
-          <t>DATA-02</t>
+          <t>DATA-02,GRADE-01</t>
         </is>
       </c>
       <c r="I21" s="15" t="inlineStr">
         <is>
-          <t>Breakdown totals reconcile to sales.</t>
+          <t>Each sale receives a grade from its margin and days-on-hand.</t>
         </is>
       </c>
       <c r="J21" s="15" t="inlineStr">
         <is>
-          <t>Validated in POC.</t>
+          <t>Exact formula in Impl. Notes. Does NOT use market data.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>BUY-01</t>
+          <t>SALES-04</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Buy Signals &amp; Funding</t>
+          <t>Sales Analytics</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Restock (buy) signals: rank models to re-buy by a buy score derived from the business's own demand (sales velocity) and profit; brand → line → model drill-down.</t>
+          <t>Sales breakdown by brand &amp; condition: units, revenue, profit, margin.</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -1945,14 +1941,14 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>Must</t>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Should</t>
         </is>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G22" s="13" t="inlineStr">
@@ -1967,19 +1963,19 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Fast-selling, profitable models rank highest to restock.</t>
+          <t>Breakdown totals reconcile to sales.</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr">
         <is>
-          <t>Distinct from Deal Radar buy ALERTS (live market offers). This is own-history restock guidance.</t>
+          <t>Validated in POC.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="46" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>BUY-02</t>
+          <t>BUY-01</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
@@ -1989,7 +1985,7 @@
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>Funding scenarios: spread a budget across top buy-signal models (greedy allocation), showing projected cost and profit, with per-row exclude/restore.</t>
+          <t>Restock (buy) signals: rank models to re-buy by a buy score derived from the business's own demand (sales velocity) and profit; brand → line → model drill-down.</t>
         </is>
       </c>
       <c r="D23" s="15" t="inlineStr">
@@ -1997,9 +1993,9 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E23" s="18" t="inlineStr">
-        <is>
-          <t>Should</t>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="F23" s="17" t="inlineStr">
@@ -2014,24 +2010,24 @@
       </c>
       <c r="H23" s="15" t="inlineStr">
         <is>
-          <t>BUY-01</t>
+          <t>DATA-02</t>
         </is>
       </c>
       <c r="I23" s="15" t="inlineStr">
         <is>
-          <t>A budget produces an affordable, ranked shopping list.</t>
+          <t>Fast-selling, profitable models rank highest to restock.</t>
         </is>
       </c>
       <c r="J23" s="15" t="inlineStr">
         <is>
-          <t>Excluding a model frees its budget; the allocation pulls in the next pick.</t>
+          <t>Distinct from Deal Radar buy ALERTS (live market offers). This is own-history restock guidance.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="46" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>BUY-03</t>
+          <t>BUY-02</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
@@ -2041,7 +2037,7 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Watches-to-sell list: items to move first, worst quality grade first, then most capital tied up.</t>
+          <t>Funding scenarios: spread a budget across top buy-signal models (greedy allocation), showing projected cost and profit, with per-row exclude/restore.</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2049,14 +2045,14 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
-        <is>
-          <t>Must</t>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Should</t>
         </is>
       </c>
       <c r="F24" s="13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G24" s="13" t="inlineStr">
@@ -2066,34 +2062,34 @@
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>INV-03</t>
+          <t>BUY-01</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Aged, high-cost stock surfaces at the top.</t>
+          <t>A budget produces an affordable, ranked shopping list.</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr">
         <is>
-          <t>Validated in POC.</t>
+          <t>Excluding a model frees its budget; the allocation pulls in the next pick.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>PROJ-01</t>
+          <t>BUY-03</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>Projections</t>
+          <t>Buy Signals &amp; Funding</t>
         </is>
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>Projected profit: target wholesale minus cost across the priced inventory.</t>
+          <t>Watches-to-sell list: items to move first, worst quality grade first, then most capital tied up.</t>
         </is>
       </c>
       <c r="D25" s="15" t="inlineStr">
@@ -2101,14 +2097,14 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E25" s="18" t="inlineStr">
-        <is>
-          <t>Should</t>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="F25" s="17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G25" s="17" t="inlineStr">
@@ -2118,24 +2114,24 @@
       </c>
       <c r="H25" s="15" t="inlineStr">
         <is>
-          <t>DATA-01</t>
+          <t>INV-03</t>
         </is>
       </c>
       <c r="I25" s="15" t="inlineStr">
         <is>
-          <t>Projected profit sums over items with a target price.</t>
+          <t>Aged, high-cost stock surfaces at the top.</t>
         </is>
       </c>
       <c r="J25" s="15" t="inlineStr">
         <is>
-          <t>Only the target-priced portion counts.</t>
+          <t>Validated in POC.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="46" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>PROJ-02</t>
+          <t>PROJ-01</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -2145,7 +2141,7 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Projected vs historical profit by model and by brand: does the projected margin match what history actually achieved.</t>
+          <t>Projected profit: target wholesale minus cost across the priced inventory.</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2153,7 +2149,7 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E26" s="19" t="inlineStr">
+      <c r="E26" s="18" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
@@ -2170,34 +2166,34 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>DATA-01,DATA-02</t>
+          <t>DATA-01</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Each model/brand shows projected vs realized margin.</t>
+          <t>Projected profit sums over items with a target price.</t>
         </is>
       </c>
       <c r="J26" s="11" t="inlineStr">
         <is>
-          <t>Validated in POC.</t>
+          <t>Only the target-priced portion counts.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="46" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>LIAB-01</t>
+          <t>PROJ-02</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>Liabilities</t>
+          <t>Projections</t>
         </is>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>Unpaid inventory liability: amount owed on inventory not yet paid for.</t>
+          <t>Projected vs historical profit by model and by brand: does the projected margin match what history actually achieved.</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
@@ -2205,9 +2201,9 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
-        <is>
-          <t>Must</t>
+      <c r="E27" s="19" t="inlineStr">
+        <is>
+          <t>Should</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
@@ -2222,24 +2218,24 @@
       </c>
       <c r="H27" s="15" t="inlineStr">
         <is>
-          <t>DATA-01</t>
+          <t>DATA-01,DATA-02</t>
         </is>
       </c>
       <c r="I27" s="15" t="inlineStr">
         <is>
-          <t>Unpaid total matches unpaid items' balances.</t>
+          <t>Each model/brand shows projected vs realized margin.</t>
         </is>
       </c>
       <c r="J27" s="15" t="inlineStr">
         <is>
-          <t>Reflects full dataset; ignores brand/period filters.</t>
+          <t>Validated in POC.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="46" customHeight="1">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>LIAB-02</t>
+          <t>LIAB-01</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -2249,7 +2245,7 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Consignment &amp; memo liability: value held on consignment or memo.</t>
+          <t>Unpaid inventory liability: amount owed on inventory not yet paid for.</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2279,15 +2275,19 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Consignment/memo total matches those items.</t>
-        </is>
-      </c>
-      <c r="J28" s="11" t="inlineStr"/>
+          <t>Unpaid total matches unpaid items' balances.</t>
+        </is>
+      </c>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>Reflects full dataset; ignores brand/period filters.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="46" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>LIAB-03</t>
+          <t>LIAB-02</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>Overpaid invoices: invoices with a negative balance (paid more than owed).</t>
+          <t>Consignment &amp; memo liability: value held on consignment or memo.</t>
         </is>
       </c>
       <c r="D29" s="15" t="inlineStr">
@@ -2305,9 +2305,9 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E29" s="18" t="inlineStr">
-        <is>
-          <t>Should</t>
+      <c r="E29" s="16" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="I29" s="15" t="inlineStr">
         <is>
-          <t>Negative-balance invoices are listed and totalled.</t>
+          <t>Consignment/memo total matches those items.</t>
         </is>
       </c>
       <c r="J29" s="15" t="inlineStr"/>
@@ -2335,7 +2335,7 @@
     <row r="30" ht="46" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>LIAB-04</t>
+          <t>LIAB-03</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Estimated sales tax by state.</t>
+          <t>Overpaid invoices: invoices with a negative balance (paid more than owed).</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2353,7 +2353,7 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E30" s="19" t="inlineStr">
+      <c r="E30" s="18" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
@@ -2370,42 +2370,38 @@
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>DATA-02</t>
+          <t>DATA-01</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Tax estimate groups by state.</t>
-        </is>
-      </c>
-      <c r="J30" s="11" t="inlineStr">
-        <is>
-          <t>Validated in POC.</t>
-        </is>
-      </c>
+          <t>Negative-balance invoices are listed and totalled.</t>
+        </is>
+      </c>
+      <c r="J30" s="11" t="inlineStr"/>
     </row>
     <row r="31" ht="46" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>GRADE-01</t>
+          <t>LIAB-04</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>Grading &amp; Config</t>
+          <t>Liabilities</t>
         </is>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>The DJ sales grade shall be per-business configurable: margin-vs-velocity weighting, factor thresholds, and harshness. Set by the admin tier; applies business-wide.</t>
+          <t>Estimated sales tax by state.</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>Admin tier</t>
-        </is>
-      </c>
-      <c r="E31" s="18" t="inlineStr">
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E31" s="19" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
@@ -2422,24 +2418,24 @@
       </c>
       <c r="H31" s="15" t="inlineStr">
         <is>
-          <t>SALES-03,PLAT-04</t>
+          <t>DATA-02</t>
         </is>
       </c>
       <c r="I31" s="15" t="inlineStr">
         <is>
-          <t>Changing weights re-grades all sales consistently.</t>
+          <t>Tax estimate groups by state.</t>
         </is>
       </c>
       <c r="J31" s="15" t="inlineStr">
         <is>
-          <t>Formula in Impl. Notes.</t>
+          <t>Validated in POC.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="46" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>GRADE-02</t>
+          <t>GRADE-01</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
@@ -2449,7 +2445,7 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>The inventory aging grade thresholds (days → A–F) shall be per-business configurable by the admin tier.</t>
+          <t>The DJ sales grade shall be per-business configurable: margin-vs-velocity weighting, factor thresholds, and harshness. Set by the admin tier; applies business-wide.</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2457,7 +2453,7 @@
           <t>Admin tier</t>
         </is>
       </c>
-      <c r="E32" s="19" t="inlineStr">
+      <c r="E32" s="18" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
@@ -2474,45 +2470,49 @@
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>INV-03</t>
+          <t>SALES-03,PLAT-04</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Changing thresholds re-buckets inventory.</t>
-        </is>
-      </c>
-      <c r="J32" s="11" t="inlineStr"/>
+          <t>Changing weights re-grades all sales consistently.</t>
+        </is>
+      </c>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t>Formula in Impl. Notes.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="46" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>UI-01</t>
+          <t>GRADE-02</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>Detail &amp; UI</t>
+          <t>Grading &amp; Config</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>Present four tabs: Inventory, Sales, Buy Signals, Liabilities. (Alerts is the separate Deal Radar feature.)</t>
+          <t>The inventory aging grade thresholds (days → A–F) shall be per-business configurable by the admin tier.</t>
         </is>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>All</t>
-        </is>
-      </c>
-      <c r="E33" s="16" t="inlineStr">
-        <is>
-          <t>Must</t>
+          <t>Admin tier</t>
+        </is>
+      </c>
+      <c r="E33" s="19" t="inlineStr">
+        <is>
+          <t>Should</t>
         </is>
       </c>
       <c r="F33" s="17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G33" s="17" t="inlineStr">
@@ -2520,10 +2520,14 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="H33" s="15" t="inlineStr"/>
+      <c r="H33" s="15" t="inlineStr">
+        <is>
+          <t>INV-03</t>
+        </is>
+      </c>
       <c r="I33" s="15" t="inlineStr">
         <is>
-          <t>The four tabs render their respective analytics.</t>
+          <t>Changing thresholds re-buckets inventory.</t>
         </is>
       </c>
       <c r="J33" s="15" t="inlineStr"/>
@@ -2531,7 +2535,7 @@
     <row r="34" ht="46" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>UI-02</t>
+          <t>UI-01</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
@@ -2541,7 +2545,7 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Global filters (brand, status, period) apply across analytic views; liabilities intentionally ignore filters and show full exposure.</t>
+          <t>Present four tabs: Inventory, Sales, Buy Signals, Liabilities. (Alerts is the separate Deal Radar feature.)</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2549,9 +2553,9 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E34" s="19" t="inlineStr">
-        <is>
-          <t>Should</t>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="F34" s="13" t="inlineStr">
@@ -2567,19 +2571,15 @@
       <c r="H34" s="11" t="inlineStr"/>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Filtering brand narrows analytics but not liabilities.</t>
-        </is>
-      </c>
-      <c r="J34" s="11" t="inlineStr">
-        <is>
-          <t>Liabilities = real financial exposure, always full.</t>
-        </is>
-      </c>
+          <t>The four tabs render their respective analytics.</t>
+        </is>
+      </c>
+      <c r="J34" s="11" t="inlineStr"/>
     </row>
     <row r="35" ht="46" customHeight="1">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>UI-03</t>
+          <t>UI-02</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>Click-through drill-down throughout (brand→model, salesperson→sales, model→its items).</t>
+          <t>Global filters (brand, status, period) apply across analytic views; liabilities intentionally ignore filters and show full exposure.</t>
         </is>
       </c>
       <c r="D35" s="15" t="inlineStr">
@@ -2597,7 +2597,7 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E35" s="18" t="inlineStr">
+      <c r="E35" s="19" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
@@ -2615,15 +2615,19 @@
       <c r="H35" s="15" t="inlineStr"/>
       <c r="I35" s="15" t="inlineStr">
         <is>
-          <t>Clicking a summary row reveals its detail.</t>
-        </is>
-      </c>
-      <c r="J35" s="15" t="inlineStr"/>
+          <t>Filtering brand narrows analytics but not liabilities.</t>
+        </is>
+      </c>
+      <c r="J35" s="15" t="inlineStr">
+        <is>
+          <t>Liabilities = real financial exposure, always full.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="46" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>UI-04</t>
+          <t>UI-03</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
@@ -2633,7 +2637,7 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Within an analysis (e.g. funding scenarios), a user may exclude/adjust items and restore them; the change affects that view.</t>
+          <t>Click-through drill-down throughout (brand→model, salesperson→sales, model→its items).</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -2641,14 +2645,14 @@
           <t>All</t>
         </is>
       </c>
-      <c r="E36" s="19" t="inlineStr">
+      <c r="E36" s="18" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G36" s="13" t="inlineStr">
@@ -2656,74 +2660,70 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="H36" s="11" t="inlineStr">
-        <is>
-          <t>BUY-02</t>
-        </is>
-      </c>
+      <c r="H36" s="11" t="inlineStr"/>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Excluding an item updates the analysis and is restorable.</t>
-        </is>
-      </c>
-      <c r="J36" s="11" t="inlineStr">
-        <is>
-          <t>Saved/shared config is admin-tier; ad-hoc view tweaks are per-user.</t>
-        </is>
-      </c>
+          <t>Clicking a summary row reveals its detail.</t>
+        </is>
+      </c>
+      <c r="J36" s="11" t="inlineStr"/>
     </row>
     <row r="37" ht="46" customHeight="1">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>NFR-01</t>
+          <t>UI-04</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>Non-Functional</t>
+          <t>Detail &amp; UI</t>
         </is>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>Strict multi-tenant isolation of inventory, sales, config, and derived analytics between businesses.</t>
+          <t>Within an analysis (e.g. funding scenarios), a user may exclude/adjust items and restore them; the change affects that view.</t>
         </is>
       </c>
       <c r="D37" s="15" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E37" s="16" t="inlineStr">
-        <is>
-          <t>Must</t>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>Should</t>
         </is>
       </c>
       <c r="F37" s="17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G37" s="17" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="H37" s="15" t="inlineStr">
         <is>
-          <t>PLAT-04</t>
+          <t>BUY-02</t>
         </is>
       </c>
       <c r="I37" s="15" t="inlineStr">
         <is>
-          <t>No cross-business data access by any path.</t>
-        </is>
-      </c>
-      <c r="J37" s="15" t="inlineStr"/>
+          <t>Excluding an item updates the analysis and is restorable.</t>
+        </is>
+      </c>
+      <c r="J37" s="15" t="inlineStr">
+        <is>
+          <t>Saved/shared config is admin-tier; ad-hoc view tweaks are per-user.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="46" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>NFR-02</t>
+          <t>NFR-01</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Compute analytics over a business's full inventory and sales within a responsive budget (caching / incremental where needed).</t>
+          <t>Strict multi-tenant isolation of inventory, sales, config, and derived analytics between businesses.</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -2741,87 +2741,135 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E38" s="19" t="inlineStr">
-        <is>
-          <t>Should</t>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="F38" s="13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="H38" s="11" t="inlineStr"/>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="inlineStr">
+        <is>
+          <t>PLAT-04</t>
+        </is>
+      </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Dashboard loads and recomputes within an acceptable time.</t>
-        </is>
-      </c>
-      <c r="J38" s="11" t="inlineStr">
-        <is>
-          <t>POC caches the WatchOps pulls.</t>
-        </is>
-      </c>
+          <t>No cross-business data access by any path.</t>
+        </is>
+      </c>
+      <c r="J38" s="11" t="inlineStr"/>
     </row>
     <row r="39" ht="46" customHeight="1">
       <c r="A39" s="14" t="inlineStr">
         <is>
+          <t>NFR-02</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>Non-Functional</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>Compute analytics over a business's full inventory and sales within a responsive budget (caching / incremental where needed).</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E39" s="19" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="F39" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G39" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H39" s="15" t="inlineStr"/>
+      <c r="I39" s="15" t="inlineStr">
+        <is>
+          <t>Dashboard loads and recomputes within an acceptable time.</t>
+        </is>
+      </c>
+      <c r="J39" s="15" t="inlineStr">
+        <is>
+          <t>POC caches the WatchOps pulls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="46" customHeight="1">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
           <t>NFR-03</t>
         </is>
       </c>
-      <c r="B39" s="15" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>Non-Functional</t>
         </is>
       </c>
-      <c r="C39" s="15" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>Handle WatchOps inventory pagination, exclude voided/sold items, and map inventory types (owned / memo / partnership / consignment) correctly.</t>
         </is>
       </c>
-      <c r="D39" s="15" t="inlineStr">
+      <c r="D40" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E39" s="16" t="inlineStr">
+      <c r="E40" s="12" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F39" s="17" t="inlineStr">
+      <c r="F40" s="13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G39" s="17" t="inlineStr">
+      <c r="G40" s="13" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H39" s="15" t="inlineStr">
+      <c r="H40" s="11" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="I39" s="15" t="inlineStr">
+      <c r="I40" s="11" t="inlineStr">
         <is>
           <t>All live holdings load; voids/sold excluded; types correct.</t>
         </is>
       </c>
-      <c r="J39" s="15" t="inlineStr">
+      <c r="J40" s="11" t="inlineStr">
         <is>
           <t>Validated in POC.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J39"/>
+  <autoFilter ref="A1:J40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3232,7 +3280,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Whether the dashboard should support a book imported from Sheet/API for businesses not on WatchOps (as Deal Radar allows). Out of scope unless needed.</t>
+          <t>Excel/CSV upload (DATA-05) already lets a non-WatchOps business use the dashboard. A live Google-Sheet/API connector (auto-refreshing, vs a one-off upload) is the remaining open question.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reword requirements in plain, self-contained language
Rewrote every requirement and acceptance criterion to stand on its own for the
WatchOps devs: defines terms inline (velocity, weeks-of-stock, aging grade, the
DJ per-sale grade, consignment/memo, projected profit) and explains why where it
aids comprehension. Same 39 requirements, same IDs and priorities; clearer,
longer wording only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WatchBI_Dashboard_Requirements.xlsx
+++ b/WatchBI_Dashboard_Requirements.xlsx
@@ -912,7 +912,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="46" customHeight="1">
+    <row r="2" ht="52" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
           <t>PLAT-01</t>
@@ -925,7 +925,7 @@
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>The dashboard shall operate as a licensed feature inside WatchOps, gated by a paid entitlement.</t>
+          <t>The dashboard shall be available only to WatchOps businesses that hold a paid entitlement for it; a business without the entitlement cannot open it.</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -951,7 +951,7 @@
       <c r="H2" s="11" t="inlineStr"/>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>No entitlement → no access; with it, the feature loads.</t>
+          <t>A business without the dashboard entitlement is blocked; a business with it can open the dashboard.</t>
         </is>
       </c>
       <c r="J2" s="11" t="inlineStr">
@@ -960,7 +960,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="46" customHeight="1">
+    <row r="3" ht="52" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
           <t>PLAT-02</t>
@@ -973,7 +973,7 @@
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
-          <t>Authenticate users through WatchOps with no separate login.</t>
+          <t>A user already signed in to WatchOps shall use the dashboard without a separate login; it relies on WatchOps for authentication.</t>
         </is>
       </c>
       <c r="D3" s="15" t="inlineStr">
@@ -999,12 +999,12 @@
       <c r="H3" s="15" t="inlineStr"/>
       <c r="I3" s="15" t="inlineStr">
         <is>
-          <t>A signed-in WatchOps user opens the dashboard without re-auth.</t>
+          <t>A signed-in WatchOps user opens the dashboard without re-entering credentials.</t>
         </is>
       </c>
       <c r="J3" s="15" t="inlineStr"/>
     </row>
-    <row r="4" ht="46" customHeight="1">
+    <row r="4" ht="52" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
           <t>PLAT-03</t>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Use WatchOps' existing businesses, users, and roles; do not define an identity model.</t>
+          <t>The dashboard shall use the businesses, users, and roles that already exist in WatchOps, and shall not maintain its own.</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1043,7 +1043,7 @@
       <c r="H4" s="11" t="inlineStr"/>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Roster and roles match WatchOps.</t>
+          <t>Users and roles match WatchOps, with no separate dashboard account list.</t>
         </is>
       </c>
       <c r="J4" s="11" t="inlineStr">
@@ -1052,7 +1052,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="46" customHeight="1">
+    <row r="5" ht="52" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
           <t>PLAT-04</t>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Persist dashboard state (grading config, saved filters/exclusions) in the platform database, isolated per business.</t>
+          <t>Any settings the dashboard stores — grading configuration, saved filters, saved exclusions — shall be kept in the WatchOps platform database, isolated per business.</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
@@ -1091,12 +1091,12 @@
       <c r="H5" s="15" t="inlineStr"/>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>Business A cannot read Business B's config or data.</t>
+          <t>One business's saved configuration cannot be read by another business.</t>
         </is>
       </c>
       <c r="J5" s="15" t="inlineStr"/>
     </row>
-    <row r="6" ht="46" customHeight="1">
+    <row r="6" ht="78" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
           <t>PLAT-05</t>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>All users in a business may view ALL analytics — cost, margin, liabilities, and every salesperson's performance. No role-based financial redaction.</t>
+          <t>Every user in a business shall be able to view all of the dashboard's analytics, including cost basis, profit margins, financial liabilities, and every salesperson's performance. No figures are hidden based on a user's role; roles only control who may change configuration.</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>A Sales Personnel Viewer sees the same numbers as an Administrator.</t>
+          <t>A Sales Personnel Viewer sees the same financial figures as an Administrator.</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
@@ -1148,7 +1148,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="46" customHeight="1">
+    <row r="7" ht="91" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
           <t>DATA-01</t>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Read the business's live inventory from the WatchOps API (default): cost, target prices, condition, status, inventory type, supplier, serial, payment status, purchase date; OR from an uploaded inventory sheet (see DATA-05).</t>
+          <t>The dashboard shall read the business's current inventory from the WatchOps API by default — including each item's cost, target prices, condition, status, inventory type, supplier, serial number, payment status, and purchase date — or, alternatively, from an uploaded inventory spreadsheet (see DATA-05).</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>Inventory analytics reflect current WatchOps holdings, or the uploaded sheet.</t>
+          <t>Inventory analytics reflect the current WatchOps holdings, or the uploaded sheet when one is used.</t>
         </is>
       </c>
       <c r="J7" s="15" t="inlineStr">
@@ -1200,7 +1200,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="46" customHeight="1">
+    <row r="8" ht="65" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
           <t>DATA-02</t>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Read sales history from the WatchOps API (default): sold items with sold price, cost, condition, salesperson, and dates; OR from an uploaded sales sheet (see DATA-05).</t>
+          <t>The dashboard shall read the business's sales history from the WatchOps API by default — each sold item's sale price, cost, condition, salesperson, and dates — or, alternatively, from an uploaded sales spreadsheet (see DATA-05).</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Sales analytics reflect WatchOps sales, or the uploaded sheet.</t>
+          <t>Sales analytics reflect WatchOps sales, or the uploaded sheet when one is used.</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
@@ -1252,7 +1252,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="46" customHeight="1">
+    <row r="9" ht="65" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
           <t>DATA-03</t>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>No external market-value data. WatchCharts is removed; any view comparing to market value is out of scope for v1.</t>
+          <t>The dashboard shall not depend on any external market-value data. The previous WatchCharts integration is removed, and every view that compared the business's prices to open-market value is out of scope for the first version.</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -1291,7 +1291,7 @@
       <c r="H9" s="15" t="inlineStr"/>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>No dashboard view depends on an external market API.</t>
+          <t>No dashboard view requires an external market-data source in order to render.</t>
         </is>
       </c>
       <c r="J9" s="15" t="inlineStr">
@@ -1300,7 +1300,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="46" customHeight="1">
+    <row r="10" ht="78" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
           <t>DATA-04</t>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Decode WatchOps numeric codes to text correctly (condition, inventory status, box/papers) before any analytic uses them.</t>
+          <t>Before any analytic uses them, the dashboard shall translate WatchOps' numeric codes into their correct text meanings — for condition, inventory status, and box/papers — using the verified code legends (see Implementation Notes; an earlier version had the condition mapping reversed).</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Condition/status labels match the WatchOps export exactly.</t>
+          <t>Condition and status labels shown in the dashboard match the WatchOps export exactly.</t>
         </is>
       </c>
       <c r="J10" s="11" t="inlineStr">
@@ -1352,7 +1352,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="46" customHeight="1">
+    <row r="11" ht="91" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
           <t>DATA-05</t>
@@ -1365,7 +1365,7 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>Support uploading inventory and/or sales history via Excel/CSV, as an alternative or supplement to the WatchOps API. The importer shall detect the sheet's columns and let the user confirm the field mapping, so it works with any dealer's export format.</t>
+          <t>The dashboard shall let a user upload inventory and/or sales history as an Excel or CSV file, either instead of or in addition to the WatchOps API. Because dealers' spreadsheets differ, the importer shall detect the file's columns and let the user confirm which column maps to which field, so it works with any export format.</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
@@ -1400,7 +1400,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="46" customHeight="1">
+    <row r="12" ht="78" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>INV-01</t>
@@ -1413,7 +1413,7 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Inventory KPI header: items in stock, capital tied up, count aged 91+ days, median days to sell, overall health.</t>
+          <t>The Inventory view shall show a header of key figures: the number of items in stock, the total capital tied up in them, how many have been in stock for 91 days or more, the median number of days to sell, and an overall inventory-health indicator.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Header figures match the underlying inventory.</t>
+          <t>The header figures reconcile with the underlying inventory.</t>
         </is>
       </c>
       <c r="J12" s="11" t="inlineStr">
@@ -1452,7 +1452,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="46" customHeight="1">
+    <row r="13" ht="65" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
           <t>INV-02</t>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>Inventory breakdowns: by brand, by brand &amp; condition (new/used), by inventory type (owned/memo/partnership/consignment), by price tier, by product line, and by model number.</t>
+          <t>The Inventory view shall break the stock down several ways: by brand; by brand and condition (new versus used); by inventory type (owned, memo, partnership, consignment); by price tier; by product line; and by model number.</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>Each breakdown totals to the inventory.</t>
+          <t>Each breakdown's totals add up to the full inventory.</t>
         </is>
       </c>
       <c r="J13" s="15" t="inlineStr">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="46" customHeight="1">
+    <row r="14" ht="65" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
           <t>INV-03</t>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Inventory aging: age buckets and an A→F quality grade (A = fresh, F = aged) based on days in stock.</t>
+          <t>The dashboard shall show how aged the inventory is — grouping items into age buckets and assigning each an A-to-F quality grade based on days in stock, where A is fresh and F is heavily aged.</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>Each item lands in the correct age bucket / grade.</t>
+          <t>Each item falls into the correct age bucket and quality grade.</t>
         </is>
       </c>
       <c r="J14" s="11" t="inlineStr">
@@ -1556,7 +1556,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="46" customHeight="1">
+    <row r="15" ht="65" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
           <t>INV-04</t>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>Sell-through velocity: weekly velocity and weeks-of-stock per model and brand, from recent sales.</t>
+          <t>The dashboard shall compute sell-through velocity — how quickly stock moves — expressed as a weekly sales rate and as 'weeks of stock on hand', for each model and brand, based on recent sales.</t>
         </is>
       </c>
       <c r="D15" s="15" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>Velocity and weeks-of-stock compute per model/brand.</t>
+          <t>Velocity and weeks-of-stock are computed for each model and brand.</t>
         </is>
       </c>
       <c r="J15" s="15" t="inlineStr">
@@ -1608,7 +1608,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="46" customHeight="1">
+    <row r="16" ht="52" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
           <t>INV-05</t>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Supplier view: spend, units, and aging by supplier (top suppliers).</t>
+          <t>The dashboard shall provide a supplier view showing spend, unit count, and aging grouped by supplier (top suppliers).</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>Supplier totals reconcile to inventory.</t>
+          <t>Supplier totals reconcile with the inventory.</t>
         </is>
       </c>
       <c r="J16" s="11" t="inlineStr">
@@ -1660,7 +1660,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="46" customHeight="1">
+    <row r="17" ht="65" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
           <t>INV-06</t>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>Data-quality view: flag inventory with missing/blank key fields (no brand and no model, missing cost, etc.).</t>
+          <t>The dashboard shall provide a data-quality view that flags inventory records missing key fields — for example an item with neither a brand nor a model name, or with no cost recorded.</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>Rows with missing fields are listed and counted.</t>
+          <t>Records with missing key fields are listed and counted.</t>
         </is>
       </c>
       <c r="J17" s="15" t="inlineStr">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="46" customHeight="1">
+    <row r="18" ht="52" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
           <t>INV-07</t>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Drill-down navigation: brand → product line → model.</t>
+          <t>The dashboard shall let the user drill down from a brand into its product lines, and from a line into individual models.</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>Clicking a brand narrows to its lines and models.</t>
+          <t>Clicking a brand reveals its lines, and clicking a line reveals its models.</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr">
@@ -1764,7 +1764,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="46" customHeight="1">
+    <row r="19" ht="52" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
           <t>SALES-01</t>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>Sales KPI header: revenue, units sold, total profit $, median margin %.</t>
+          <t>The Sales view shall show a header of key figures: total revenue, units sold, total profit in dollars, and the median profit-margin percentage.</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
-          <t>Header figures match the sales set.</t>
+          <t>The header figures reconcile with the sales set.</t>
         </is>
       </c>
       <c r="J19" s="15" t="inlineStr">
@@ -1816,7 +1816,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="46" customHeight="1">
+    <row r="20" ht="65" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
           <t>SALES-02</t>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Salesperson performance: profit, units, and velocity (median days to sell) per salesperson, with drill-down into each sale.</t>
+          <t>The Sales view shall show each salesperson's performance — profit, units sold, and selling velocity (median days to sell) — and shall let the user drill into that salesperson's individual sales.</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>Each salesperson's totals reconcile; sales are drillable.</t>
+          <t>Each salesperson's totals reconcile, and their individual sales can be viewed.</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
@@ -1868,7 +1868,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="46" customHeight="1">
+    <row r="21" ht="91" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
           <t>SALES-03</t>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>Per-sale performance grade (the DJ grade): a points system over margin and velocity (days on hand), grade A–D.</t>
+          <t>The dashboard shall assign each individual sale a performance grade (A to D) using a points system based on the profit margin and how quickly the item sold (days on hand). This grade uses only the business's own figures — no external market data. The exact formula is in the Implementation Notes tab.</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="I21" s="15" t="inlineStr">
         <is>
-          <t>Each sale receives a grade from its margin and days-on-hand.</t>
+          <t>Each sale receives a grade derived from its margin and its days-on-hand.</t>
         </is>
       </c>
       <c r="J21" s="15" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Sales breakdown by brand &amp; condition: units, revenue, profit, margin.</t>
+          <t>The Sales view shall break sales down by brand and condition, showing units, revenue, profit, and margin.</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Breakdown totals reconcile to sales.</t>
+          <t>The breakdown's totals reconcile with total sales.</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr">
@@ -1972,7 +1972,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="46" customHeight="1">
+    <row r="23" ht="104" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
           <t>BUY-01</t>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>Restock (buy) signals: rank models to re-buy by a buy score derived from the business's own demand (sales velocity) and profit; brand → line → model drill-down.</t>
+          <t>The dashboard shall recommend which models to re-buy (restock), ranking them by a buy score computed from the business's own demand (how fast the model sells) and its profitability, with drill-down from brand to line to model. This is guidance from the business's own sales history — distinct from Deal Radar's live buy alerts, which come from dealer messages.</t>
         </is>
       </c>
       <c r="D23" s="15" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="I23" s="15" t="inlineStr">
         <is>
-          <t>Fast-selling, profitable models rank highest to restock.</t>
+          <t>Fast-selling, profitable models rank highest in the restock recommendations.</t>
         </is>
       </c>
       <c r="J23" s="15" t="inlineStr">
@@ -2024,7 +2024,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="46" customHeight="1">
+    <row r="24" ht="91" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
           <t>BUY-02</t>
@@ -2037,7 +2037,7 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Funding scenarios: spread a budget across top buy-signal models (greedy allocation), showing projected cost and profit, with per-row exclude/restore.</t>
+          <t>The dashboard shall provide a funding-scenario tool: given a budget, it spreads that budget across the top restock candidates (filling the budget greedily), shows the projected cost and profit, and lets the user exclude individual models — which frees their budget for the next candidates — with the ability to restore them.</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>A budget produces an affordable, ranked shopping list.</t>
+          <t>A budget produces a ranked, affordable shopping list; excluding an item frees its budget and pulls in the next pick.</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr">
@@ -2076,7 +2076,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="46" customHeight="1">
+    <row r="25" ht="52" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
           <t>BUY-03</t>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>Watches-to-sell list: items to move first, worst quality grade first, then most capital tied up.</t>
+          <t>The dashboard shall provide a 'watches to sell' list that highlights which items to move first — worst inventory grade first, then the items with the most capital tied up.</t>
         </is>
       </c>
       <c r="D25" s="15" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="I25" s="15" t="inlineStr">
         <is>
-          <t>Aged, high-cost stock surfaces at the top.</t>
+          <t>Aged, high-cost stock appears at the top of the list.</t>
         </is>
       </c>
       <c r="J25" s="15" t="inlineStr">
@@ -2128,7 +2128,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="46" customHeight="1">
+    <row r="26" ht="52" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
           <t>PROJ-01</t>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Projected profit: target wholesale minus cost across the priced inventory.</t>
+          <t>The dashboard shall show projected profit — the target wholesale price minus cost — summed across the inventory that has a target price set.</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Projected profit sums over items with a target price.</t>
+          <t>Projected profit sums correctly over the items that have a target price.</t>
         </is>
       </c>
       <c r="J26" s="11" t="inlineStr">
@@ -2180,7 +2180,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="46" customHeight="1">
+    <row r="27" ht="65" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
           <t>PROJ-02</t>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>Projected vs historical profit by model and by brand: does the projected margin match what history actually achieved.</t>
+          <t>The dashboard shall compare projected profit against historically realized profit, by model and by brand, so the user can see whether projected margins line up with what the business has actually achieved.</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="I27" s="15" t="inlineStr">
         <is>
-          <t>Each model/brand shows projected vs realized margin.</t>
+          <t>Each model and brand shows its projected margin alongside its historically realized margin.</t>
         </is>
       </c>
       <c r="J27" s="15" t="inlineStr">
@@ -2232,7 +2232,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="46" customHeight="1">
+    <row r="28" ht="52" customHeight="1">
       <c r="A28" s="10" t="inlineStr">
         <is>
           <t>LIAB-01</t>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Unpaid inventory liability: amount owed on inventory not yet paid for.</t>
+          <t>The dashboard shall show the unpaid-inventory liability — the total the business still owes on inventory it has not yet paid for.</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Unpaid total matches unpaid items' balances.</t>
+          <t>The unpaid total matches the outstanding balances of the unpaid items.</t>
         </is>
       </c>
       <c r="J28" s="11" t="inlineStr">
@@ -2284,7 +2284,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="46" customHeight="1">
+    <row r="29" ht="52" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
           <t>LIAB-02</t>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>Consignment &amp; memo liability: value held on consignment or memo.</t>
+          <t>The dashboard shall show consignment and memo liability — the value of goods the business holds on consignment or on memo, which it does not own outright.</t>
         </is>
       </c>
       <c r="D29" s="15" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="I29" s="15" t="inlineStr">
         <is>
-          <t>Consignment/memo total matches those items.</t>
+          <t>The consignment and memo total matches those items.</t>
         </is>
       </c>
       <c r="J29" s="15" t="inlineStr"/>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Overpaid invoices: invoices with a negative balance (paid more than owed).</t>
+          <t>The dashboard shall list overpaid invoices — invoices with a negative balance, where more was paid than was owed.</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Negative-balance invoices are listed and totalled.</t>
+          <t>Invoices with a negative balance are listed and totalled.</t>
         </is>
       </c>
       <c r="J30" s="11" t="inlineStr"/>
@@ -2393,7 +2393,7 @@
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>Estimated sales tax by state.</t>
+          <t>The dashboard shall show an estimate of sales tax owed, grouped by state.</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="I31" s="15" t="inlineStr">
         <is>
-          <t>Tax estimate groups by state.</t>
+          <t>The sales-tax estimate is grouped by state.</t>
         </is>
       </c>
       <c r="J31" s="15" t="inlineStr">
@@ -2432,7 +2432,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="46" customHeight="1">
+    <row r="32" ht="78" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
         <is>
           <t>GRADE-01</t>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>The DJ sales grade shall be per-business configurable: margin-vs-velocity weighting, factor thresholds, and harshness. Set by the admin tier; applies business-wide.</t>
+          <t>The per-sale performance grade shall be tunable per business: a user in the admin tier can adjust how much margin versus selling speed counts, the thresholds for each, and the overall harshness. The chosen settings apply to everyone in the business.</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Changing weights re-grades all sales consistently.</t>
+          <t>Changing the weighting re-grades all of that business's sales consistently.</t>
         </is>
       </c>
       <c r="J32" s="11" t="inlineStr">
@@ -2484,7 +2484,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="46" customHeight="1">
+    <row r="33" ht="52" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
           <t>GRADE-02</t>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>The inventory aging grade thresholds (days → A–F) shall be per-business configurable by the admin tier.</t>
+          <t>The inventory aging grade shall be tunable per business: a user in the admin tier can set the day thresholds that map to grades A through F.</t>
         </is>
       </c>
       <c r="D33" s="15" t="inlineStr">
@@ -2527,12 +2527,12 @@
       </c>
       <c r="I33" s="15" t="inlineStr">
         <is>
-          <t>Changing thresholds re-buckets inventory.</t>
+          <t>Changing the day thresholds re-buckets the inventory into new grades.</t>
         </is>
       </c>
       <c r="J33" s="15" t="inlineStr"/>
     </row>
-    <row r="34" ht="46" customHeight="1">
+    <row r="34" ht="52" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
           <t>UI-01</t>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Present four tabs: Inventory, Sales, Buy Signals, Liabilities. (Alerts is the separate Deal Radar feature.)</t>
+          <t>The dashboard shall present four tabs — Inventory, Sales, Buy Signals, and Liabilities. Live dealer-message alerts are handled by the separate Deal Radar feature, not here.</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2571,12 +2571,12 @@
       <c r="H34" s="11" t="inlineStr"/>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>The four tabs render their respective analytics.</t>
+          <t>The four tabs each render their respective analytics.</t>
         </is>
       </c>
       <c r="J34" s="11" t="inlineStr"/>
     </row>
-    <row r="35" ht="46" customHeight="1">
+    <row r="35" ht="65" customHeight="1">
       <c r="A35" s="14" t="inlineStr">
         <is>
           <t>UI-02</t>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>Global filters (brand, status, period) apply across analytic views; liabilities intentionally ignore filters and show full exposure.</t>
+          <t>Global filters — brand, status, and time period — shall apply across the analytic views. The Liabilities view is a deliberate exception: it always shows full financial exposure and ignores these filters.</t>
         </is>
       </c>
       <c r="D35" s="15" t="inlineStr">
@@ -2615,7 +2615,7 @@
       <c r="H35" s="15" t="inlineStr"/>
       <c r="I35" s="15" t="inlineStr">
         <is>
-          <t>Filtering brand narrows analytics but not liabilities.</t>
+          <t>Applying a brand filter narrows the analytic views but not the liabilities figures.</t>
         </is>
       </c>
       <c r="J35" s="15" t="inlineStr">
@@ -2624,7 +2624,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="46" customHeight="1">
+    <row r="36" ht="65" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>UI-03</t>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Click-through drill-down throughout (brand→model, salesperson→sales, model→its items).</t>
+          <t>The dashboard shall support click-through drill-down throughout — for example from a brand to its models, from a salesperson to their sales, and from a model to its individual items.</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -2663,12 +2663,12 @@
       <c r="H36" s="11" t="inlineStr"/>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Clicking a summary row reveals its detail.</t>
+          <t>Clicking a summary row reveals the detail behind it.</t>
         </is>
       </c>
       <c r="J36" s="11" t="inlineStr"/>
     </row>
-    <row r="37" ht="46" customHeight="1">
+    <row r="37" ht="78" customHeight="1">
       <c r="A37" s="14" t="inlineStr">
         <is>
           <t>UI-04</t>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>Within an analysis (e.g. funding scenarios), a user may exclude/adjust items and restore them; the change affects that view.</t>
+          <t>Within an analysis such as the funding scenarios, a user shall be able to exclude or adjust items and later restore them; the change affects that analysis view. Ad-hoc view tweaks are personal to the user, while saved business-wide configuration is admin-tier.</t>
         </is>
       </c>
       <c r="D37" s="15" t="inlineStr">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="I37" s="15" t="inlineStr">
         <is>
-          <t>Excluding an item updates the analysis and is restorable.</t>
+          <t>Excluding an item updates the analysis and can be undone.</t>
         </is>
       </c>
       <c r="J37" s="15" t="inlineStr">
@@ -2720,7 +2720,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="46" customHeight="1">
+    <row r="38" ht="52" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
           <t>NFR-01</t>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Strict multi-tenant isolation of inventory, sales, config, and derived analytics between businesses.</t>
+          <t>The system shall keep each business's inventory, sales, configuration, and all derived analytics strictly isolated from every other business.</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>No cross-business data access by any path.</t>
+          <t>No path allows one business to read another business's data.</t>
         </is>
       </c>
       <c r="J38" s="11" t="inlineStr"/>
     </row>
-    <row r="39" ht="46" customHeight="1">
+    <row r="39" ht="65" customHeight="1">
       <c r="A39" s="14" t="inlineStr">
         <is>
           <t>NFR-02</t>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>Compute analytics over a business's full inventory and sales within a responsive budget (caching / incremental where needed).</t>
+          <t>The dashboard shall compute its analytics across a business's full inventory and sales history within a responsive time budget, using caching or incremental computation where needed.</t>
         </is>
       </c>
       <c r="D39" s="15" t="inlineStr">
@@ -2807,7 +2807,7 @@
       <c r="H39" s="15" t="inlineStr"/>
       <c r="I39" s="15" t="inlineStr">
         <is>
-          <t>Dashboard loads and recomputes within an acceptable time.</t>
+          <t>The dashboard loads and recomputes within an acceptable time on a full dataset.</t>
         </is>
       </c>
       <c r="J39" s="15" t="inlineStr">
@@ -2816,7 +2816,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="46" customHeight="1">
+    <row r="40" ht="65" customHeight="1">
       <c r="A40" s="10" t="inlineStr">
         <is>
           <t>NFR-03</t>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Handle WatchOps inventory pagination, exclude voided/sold items, and map inventory types (owned / memo / partnership / consignment) correctly.</t>
+          <t>When reading inventory from WatchOps, the system shall page through all records, exclude items that are sold or voided, and correctly map the inventory types (owned, memo, partnership, consignment).</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>All live holdings load; voids/sold excluded; types correct.</t>
+          <t>All live holdings load, sold and voided items are excluded, and inventory types are correctly assigned.</t>
         </is>
       </c>
       <c r="J40" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Set all Dashboard requirements to Phase 1 (reassign to Phase 2 as needed)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WatchBI_Dashboard_Requirements.xlsx
+++ b/WatchBI_Dashboard_Requirements.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17940" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requirements'!$A$1:$J$40</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
@@ -33,105 +32,123 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="20"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <i val="1"/>
-      <color rgb="00808080"/>
+      <color rgb="FF808080"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00808080"/>
+      <color rgb="FF808080"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="002F5496"/>
+      <color rgb="FF2F5496"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="002F5496"/>
+      <color rgb="FF2F5496"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00C00000"/>
+      <color rgb="FFC00000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00BF8F00"/>
+      <color rgb="FFBF8F00"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <i val="1"/>
-      <color rgb="00808080"/>
+      <color rgb="FF808080"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00548235"/>
+      <color rgb="FF548235"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="002F5496"/>
+      <color rgb="FF2F5496"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00808080"/>
+      <family val="2"/>
+      <color rgb="FF808080"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -144,17 +161,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5496"/>
+        <fgColor rgb="FF2F5496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F5FA"/>
+        <fgColor rgb="FFF2F5FA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FBFBFB"/>
+        <fgColor rgb="FFFBFBFB"/>
       </patternFill>
     </fill>
   </fills>
@@ -168,26 +185,25 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -252,18 +268,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -627,208 +646,180 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:C25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="96" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" style="27" min="1" max="1"/>
+    <col width="26" customWidth="1" style="27" min="2" max="2"/>
+    <col width="96" customWidth="1" style="27" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+    <row r="2" ht="25" customHeight="1" s="27">
+      <c r="B2" s="28" t="inlineStr">
         <is>
           <t>WatchBI Dashboard — Requirements</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="26" t="inlineStr">
         <is>
           <t>Inventory &amp; sales intelligence · a licensed feature within WatchOps · spec for the WatchOps dev team</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Prepared</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>MJ Yassine · 2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>WatchBI dashboard POC is built and running; this specifies the productized version.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+    <row r="8" ht="60" customHeight="1" s="27">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>What this is</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>An analytics dashboard over a watch dealer's own inventory and sales: aging, an A–F quality grade, sell-through velocity, a configurable per-sale performance grade, projected-vs-historical profit, restock (buy) signals with funding scenarios, and financial liabilities. It answers 'what do I hold, how fast does it move, how well are we selling it, and what do I owe.'</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="5" t="inlineStr">
+    <row r="10" ht="45" customHeight="1" s="27">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>How it ships</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>A paid feature INSIDE WatchOps, unlocked per entitlement. Not standalone. It consumes WatchOps' accounts, businesses, roles, and database. Its companion feature Deal Radar handles live dealer-message alerts (the old Alerts tab); this dashboard is the inventory/sales analytics.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="5" t="inlineStr">
+    <row r="12" ht="60" customHeight="1" s="27">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Build approach</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>GREENFIELD — the WatchOps team builds fresh; no POC code is reused. The POC is a working REFERENCE that proves the metrics and de-risks the hard parts (the WatchOps code legends, the DJ grading formula, the velocity/aging math). 'Validated in POC' in Notes means proven with a reference, not inherited. The Implementation Notes tab captures the formulas and gotchas so the fresh build reproduces them exactly.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="7" t="inlineStr">
+    <row r="14" ht="17" customHeight="1" s="27">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Decisions locked in this spec</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Identity &amp; roles</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Provided by WatchOps. Uses WatchOps login, businesses, and its five roles. See Roles &amp; Permissions.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="8" t="inlineStr">
+    <row r="16" ht="28" customHeight="1" s="27">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Financial visibility</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Everyone in the business sees ALL analytics — cost basis, margins, liabilities, and every salesperson's performance. No role-based redaction. Roles gate CONFIGURATION, not viewing.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="8" t="inlineStr">
+    <row r="17" ht="28" customHeight="1" s="27">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Data sources</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Inventory and sales history come from the WatchOps API by default. Excel/CSV upload is ALSO supported — for businesses not on WatchOps, history older than the API holds, or manual data — with flexible column mapping.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="8" t="inlineStr">
+    <row r="18" ht="28" customHeight="1" s="27">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Market data — REMOVED</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>WatchCharts (the external market-value API) is cut entirely. Every view that compared to market value (Oldest-20 / Latest-20 vs market, market-based sales grade) is OUT OF SCOPE. Everything built on the business's own data stays.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="8" t="inlineStr">
+    <row r="19" ht="28" customHeight="1" s="27">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Grading</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>The DJ sales grade (margin + velocity) and the inventory aging grade are per-business configurable by the admin tier; settings apply business-wide.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Alerts</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>The old Alerts tab is NOT part of this dashboard — it is the separate Deal Radar feature.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>How to read the Requirements tab</t>
-        </is>
-      </c>
+    <row r="22" ht="17" customHeight="1" s="27">
+      <c r="B22" s="5" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Must = v1 · Should = fast-follow · Could = backlog (MoSCoW).</t>
-        </is>
-      </c>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Provided by</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Platform (WatchOps) = an existing capability consumed · Feature (Dashboard) = new work the WatchOps devs build · Both = new logic checked against a platform capability.</t>
-        </is>
-      </c>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Acceptance criteria</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>A pass/fail check proving the requirement is met.</t>
-        </is>
-      </c>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -846,2023 +837,2023 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="38" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="11" customWidth="1" style="27" min="1" max="1"/>
+    <col width="22" customWidth="1" style="27" min="2" max="2"/>
+    <col width="62" customWidth="1" style="27" min="3" max="3"/>
+    <col width="14" customWidth="1" style="27" min="4" max="4"/>
+    <col width="10" customWidth="1" style="27" min="5" max="5"/>
+    <col width="8" customWidth="1" style="27" min="6" max="6"/>
+    <col width="14" customWidth="1" style="27" min="7" max="7"/>
+    <col width="13" customWidth="1" style="27" min="8" max="8"/>
+    <col hidden="1" width="50" customWidth="1" style="27" min="9" max="9"/>
+    <col hidden="1" width="38" customWidth="1" style="27" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="20" customHeight="1" s="27">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Provided by</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Depends on</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Acceptance criteria</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="52" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+    <row r="2" ht="52" customHeight="1" s="27">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>PLAT-01</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Platform &amp; Access</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall be available only to WatchOps businesses that hold a paid entitlement for it; a business without the entitlement cannot open it.</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F2" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G2" s="13" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H2" s="11" t="inlineStr"/>
-      <c r="I2" s="11" t="inlineStr">
+      <c r="H2" s="9" t="n"/>
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>A business without the dashboard entitlement is blocked; a business with it can open the dashboard.</t>
         </is>
       </c>
-      <c r="J2" s="11" t="inlineStr">
+      <c r="J2" s="9" t="inlineStr">
         <is>
           <t>Billing granularity TBD (Backlog).</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="52" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
+    <row r="3" ht="52" customHeight="1" s="27">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>PLAT-02</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Platform &amp; Access</t>
         </is>
       </c>
-      <c r="C3" s="15" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>A user already signed in to WatchOps shall use the dashboard without a separate login; it relies on WatchOps for authentication.</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F3" s="17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G3" s="17" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="H3" s="15" t="inlineStr"/>
-      <c r="I3" s="15" t="inlineStr">
+      <c r="H3" s="13" t="n"/>
+      <c r="I3" s="13" t="inlineStr">
         <is>
           <t>A signed-in WatchOps user opens the dashboard without re-entering credentials.</t>
         </is>
       </c>
-      <c r="J3" s="15" t="inlineStr"/>
-    </row>
-    <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="J3" s="13" t="n"/>
+    </row>
+    <row r="4" ht="52" customHeight="1" s="27">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>PLAT-03</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Platform &amp; Access</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall use the businesses, users, and roles that already exist in WatchOps, and shall not maintain its own.</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G4" s="13" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr"/>
-      <c r="I4" s="11" t="inlineStr">
+      <c r="H4" s="9" t="n"/>
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>Users and roles match WatchOps, with no separate dashboard account list.</t>
         </is>
       </c>
-      <c r="J4" s="11" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>See Roles &amp; Permissions.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+    <row r="5" ht="52" customHeight="1" s="27">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>PLAT-04</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Platform &amp; Access</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>Any settings the dashboard stores — grading configuration, saved filters, saved exclusions — shall be kept in the WatchOps platform database, isolated per business.</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E5" s="16" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F5" s="17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G5" s="17" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="H5" s="15" t="inlineStr"/>
-      <c r="I5" s="15" t="inlineStr">
+      <c r="H5" s="13" t="n"/>
+      <c r="I5" s="13" t="inlineStr">
         <is>
           <t>One business's saved configuration cannot be read by another business.</t>
         </is>
       </c>
-      <c r="J5" s="15" t="inlineStr"/>
-    </row>
-    <row r="6" ht="78" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="J5" s="13" t="n"/>
+    </row>
+    <row r="6" ht="78" customHeight="1" s="27">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>PLAT-05</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Platform &amp; Access</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Every user in a business shall be able to view all of the dashboard's analytics, including cost basis, profit margins, financial liabilities, and every salesperson's performance. No figures are hidden based on a user's role; roles only control who may change configuration.</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>PLAT-03</t>
         </is>
       </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>A Sales Personnel Viewer sees the same financial figures as an Administrator.</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>Per decision. Roles gate configuration, not viewing.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="91" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+    <row r="7" ht="91" customHeight="1" s="27">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Data Sources</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall read the business's current inventory from the WatchOps API by default — including each item's cost, target prices, condition, status, inventory type, supplier, serial number, payment status, and purchase date — or, alternatively, from an uploaded inventory spreadsheet (see DATA-05).</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F7" s="17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G7" s="17" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H7" s="15" t="inlineStr">
+      <c r="H7" s="13" t="inlineStr">
         <is>
           <t>PLAT-03</t>
         </is>
       </c>
-      <c r="I7" s="15" t="inlineStr">
+      <c r="I7" s="13" t="inlineStr">
         <is>
           <t>Inventory analytics reflect the current WatchOps holdings, or the uploaded sheet when one is used.</t>
         </is>
       </c>
-      <c r="J7" s="15" t="inlineStr">
+      <c r="J7" s="13" t="inlineStr">
         <is>
           <t>Validated in POC. Exclude sold &amp; voided items.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="65" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="8" ht="65" customHeight="1" s="27">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>DATA-02</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Data Sources</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall read the business's sales history from the WatchOps API by default — each sold item's sale price, cost, condition, salesperson, and dates — or, alternatively, from an uploaded sales spreadsheet (see DATA-05).</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>PLAT-03</t>
         </is>
       </c>
-      <c r="I8" s="11" t="inlineStr">
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t>Sales analytics reflect WatchOps sales, or the uploaded sheet when one is used.</t>
         </is>
       </c>
-      <c r="J8" s="11" t="inlineStr">
+      <c r="J8" s="9" t="inlineStr">
         <is>
           <t>API is the default; Excel upload also supported.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="65" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+    <row r="9" ht="65" customHeight="1" s="27">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>DATA-03</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Data Sources</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall not depend on any external market-value data. The previous WatchCharts integration is removed, and every view that compared the business's prices to open-market value is out of scope for the first version.</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F9" s="17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G9" s="17" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H9" s="15" t="inlineStr"/>
-      <c r="I9" s="15" t="inlineStr">
+      <c r="H9" s="13" t="n"/>
+      <c r="I9" s="13" t="inlineStr">
         <is>
           <t>No dashboard view requires an external market-data source in order to render.</t>
         </is>
       </c>
-      <c r="J9" s="15" t="inlineStr">
+      <c r="J9" s="13" t="inlineStr">
         <is>
           <t>Decision. If WatchOps adds market data later, market views can return (Backlog).</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="78" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
+    <row r="10" ht="78" customHeight="1" s="27">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>DATA-04</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Data Sources</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Before any analytic uses them, the dashboard shall translate WatchOps' numeric codes into their correct text meanings — for condition, inventory status, and box/papers — using the verified code legends (see Implementation Notes; an earlier version had the condition mapping reversed).</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="H10" s="9" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="I10" s="11" t="inlineStr">
+      <c r="I10" s="9" t="inlineStr">
         <is>
           <t>Condition and status labels shown in the dashboard match the WatchOps export exactly.</t>
         </is>
       </c>
-      <c r="J10" s="11" t="inlineStr">
+      <c r="J10" s="9" t="inlineStr">
         <is>
           <t>Legends in Implementation Notes. The old app had condition INVERTED.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="91" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+    <row r="11" ht="91" customHeight="1" s="27">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>DATA-05</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Data Sources</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall let a user upload inventory and/or sales history as an Excel or CSV file, either instead of or in addition to the WatchOps API. Because dealers' spreadsheets differ, the importer shall detect the file's columns and let the user confirm which column maps to which field, so it works with any export format.</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Admin tier</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F11" s="17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H11" s="15" t="inlineStr"/>
-      <c r="I11" s="15" t="inlineStr">
+      <c r="H11" s="13" t="n"/>
+      <c r="I11" s="13" t="inlineStr">
         <is>
           <t>A user uploads a sheet, confirms the column mapping, and the analytics populate from it.</t>
         </is>
       </c>
-      <c r="J11" s="15" t="inlineStr">
+      <c r="J11" s="13" t="inlineStr">
         <is>
           <t>Validated in POC (mapping screen). Covers non-WatchOps businesses and older history.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="78" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
+    <row r="12" ht="78" customHeight="1" s="27">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>INV-01</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Inventory Analytics</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>The Inventory view shall show a header of key figures: the number of items in stock, the total capital tied up in them, how many have been in stock for 91 days or more, the median number of days to sell, and an overall inventory-health indicator.</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G12" s="13" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="I12" s="11" t="inlineStr">
+      <c r="I12" s="9" t="inlineStr">
         <is>
           <t>The header figures reconcile with the underlying inventory.</t>
         </is>
       </c>
-      <c r="J12" s="11" t="inlineStr">
+      <c r="J12" s="9" t="inlineStr">
         <is>
           <t>Validated in POC.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="65" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
+    <row r="13" ht="65" customHeight="1" s="27">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>INV-02</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Inventory Analytics</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>The Inventory view shall break the stock down several ways: by brand; by brand and condition (new versus used); by inventory type (owned, memo, partnership, consignment); by price tier; by product line; and by model number.</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H13" s="15" t="inlineStr">
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>DATA-01,DATA-04</t>
         </is>
       </c>
-      <c r="I13" s="15" t="inlineStr">
+      <c r="I13" s="13" t="inlineStr">
         <is>
           <t>Each breakdown's totals add up to the full inventory.</t>
         </is>
       </c>
-      <c r="J13" s="15" t="inlineStr">
+      <c r="J13" s="13" t="inlineStr">
         <is>
           <t>Validated in POC.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="65" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+    <row r="14" ht="65" customHeight="1" s="27">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>INV-03</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Inventory Analytics</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall show how aged the inventory is — grouping items into age buckets and assigning each an A-to-F quality grade based on days in stock, where A is fresh and F is heavily aged.</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G14" s="13" t="inlineStr">
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H14" s="11" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="I14" s="11" t="inlineStr">
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>Each item falls into the correct age bucket and quality grade.</t>
         </is>
       </c>
-      <c r="J14" s="11" t="inlineStr">
+      <c r="J14" s="9" t="inlineStr">
         <is>
           <t>Grade thresholds configurable (GRADE-02). Formula in Impl. Notes.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="65" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
+    <row r="15" ht="65" customHeight="1" s="27">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>INV-04</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Inventory Analytics</t>
         </is>
       </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall compute sell-through velocity — how quickly stock moves — expressed as a weekly sales rate and as 'weeks of stock on hand', for each model and brand, based on recent sales.</t>
         </is>
       </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F15" s="17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G15" s="17" t="inlineStr">
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H15" s="15" t="inlineStr">
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>DATA-01,DATA-02</t>
         </is>
       </c>
-      <c r="I15" s="15" t="inlineStr">
+      <c r="I15" s="13" t="inlineStr">
         <is>
           <t>Velocity and weeks-of-stock are computed for each model and brand.</t>
         </is>
       </c>
-      <c r="J15" s="15" t="inlineStr">
+      <c r="J15" s="13" t="inlineStr">
         <is>
           <t>Sparse windows must not overstate velocity — see Impl. Notes.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="52" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="16" ht="52" customHeight="1" s="27">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>INV-05</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Inventory Analytics</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall provide a supplier view showing spend, unit count, and aging grouped by supplier (top suppliers).</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="inlineStr">
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H16" s="11" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="I16" s="11" t="inlineStr">
+      <c r="I16" s="9" t="inlineStr">
         <is>
           <t>Supplier totals reconcile with the inventory.</t>
         </is>
       </c>
-      <c r="J16" s="11" t="inlineStr">
+      <c r="J16" s="9" t="inlineStr">
         <is>
           <t>Validated in POC.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="65" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
+    <row r="17" ht="65" customHeight="1" s="27">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>INV-06</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Inventory Analytics</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall provide a data-quality view that flags inventory records missing key fields — for example an item with neither a brand nor a model name, or with no cost recorded.</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E17" s="19" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F17" s="17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G17" s="17" t="inlineStr">
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H17" s="15" t="inlineStr">
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="I17" s="15" t="inlineStr">
+      <c r="I17" s="13" t="inlineStr">
         <is>
           <t>Records with missing key fields are listed and counted.</t>
         </is>
       </c>
-      <c r="J17" s="15" t="inlineStr">
+      <c r="J17" s="13" t="inlineStr">
         <is>
           <t>Fully-blank rows filtered at source dashboard-wide.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="52" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
+    <row r="18" ht="52" customHeight="1" s="27">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>INV-07</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Inventory Analytics</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall let the user drill down from a brand into its product lines, and from a line into individual models.</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E18" s="16" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G18" s="13" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>INV-02</t>
         </is>
       </c>
-      <c r="I18" s="11" t="inlineStr">
+      <c r="I18" s="9" t="inlineStr">
         <is>
           <t>Clicking a brand reveals its lines, and clicking a line reveals its models.</t>
         </is>
       </c>
-      <c r="J18" s="11" t="inlineStr">
+      <c r="J18" s="9" t="inlineStr">
         <is>
           <t>Validated in POC.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="52" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+    <row r="19" ht="52" customHeight="1" s="27">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>SALES-01</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Sales Analytics</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C19" s="13" t="inlineStr">
         <is>
           <t>The Sales view shall show a header of key figures: total revenue, units sold, total profit in dollars, and the median profit-margin percentage.</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E19" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F19" s="17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G19" s="17" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H19" s="15" t="inlineStr">
+      <c r="H19" s="13" t="inlineStr">
         <is>
           <t>DATA-02</t>
         </is>
       </c>
-      <c r="I19" s="15" t="inlineStr">
+      <c r="I19" s="13" t="inlineStr">
         <is>
           <t>The header figures reconcile with the sales set.</t>
         </is>
       </c>
-      <c r="J19" s="15" t="inlineStr">
+      <c r="J19" s="13" t="inlineStr">
         <is>
           <t>Validated in POC.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="65" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
+    <row r="20" ht="65" customHeight="1" s="27">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>SALES-02</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Sales Analytics</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>The Sales view shall show each salesperson's performance — profit, units sold, and selling velocity (median days to sell) — and shall let the user drill into that salesperson's individual sales.</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F20" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G20" s="13" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H20" s="11" t="inlineStr">
+      <c r="H20" s="9" t="inlineStr">
         <is>
           <t>DATA-02</t>
         </is>
       </c>
-      <c r="I20" s="11" t="inlineStr">
+      <c r="I20" s="9" t="inlineStr">
         <is>
           <t>Each salesperson's totals reconcile, and their individual sales can be viewed.</t>
         </is>
       </c>
-      <c r="J20" s="11" t="inlineStr">
+      <c r="J20" s="9" t="inlineStr">
         <is>
           <t>'Everyone sees everyone' per PLAT-05.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="91" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
+    <row r="21" ht="91" customHeight="1" s="27">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>SALES-03</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Sales Analytics</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C21" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall assign each individual sale a performance grade (A to D) using a points system based on the profit margin and how quickly the item sold (days on hand). This grade uses only the business's own figures — no external market data. The exact formula is in the Implementation Notes tab.</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F21" s="17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G21" s="17" t="inlineStr">
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H21" s="15" t="inlineStr">
+      <c r="H21" s="13" t="inlineStr">
         <is>
           <t>DATA-02,GRADE-01</t>
         </is>
       </c>
-      <c r="I21" s="15" t="inlineStr">
+      <c r="I21" s="13" t="inlineStr">
         <is>
           <t>Each sale receives a grade derived from its margin and its days-on-hand.</t>
         </is>
       </c>
-      <c r="J21" s="15" t="inlineStr">
+      <c r="J21" s="13" t="inlineStr">
         <is>
           <t>Exact formula in Impl. Notes. Does NOT use market data.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="46" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="22" ht="46" customHeight="1" s="27">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>SALES-04</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Sales Analytics</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>The Sales view shall break sales down by brand and condition, showing units, revenue, profit, and margin.</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E22" s="18" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F22" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G22" s="13" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H22" s="11" t="inlineStr">
+      <c r="H22" s="9" t="inlineStr">
         <is>
           <t>DATA-02</t>
         </is>
       </c>
-      <c r="I22" s="11" t="inlineStr">
+      <c r="I22" s="9" t="inlineStr">
         <is>
           <t>The breakdown's totals reconcile with total sales.</t>
         </is>
       </c>
-      <c r="J22" s="11" t="inlineStr">
+      <c r="J22" s="9" t="inlineStr">
         <is>
           <t>Validated in POC.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="104" customHeight="1">
-      <c r="A23" s="14" t="inlineStr">
+    <row r="23" ht="104" customHeight="1" s="27">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>BUY-01</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Buy Signals &amp; Funding</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall recommend which models to re-buy (restock), ranking them by a buy score computed from the business's own demand (how fast the model sells) and its profitability, with drill-down from brand to line to model. This is guidance from the business's own sales history — distinct from Deal Radar's live buy alerts, which come from dealer messages.</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F23" s="17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G23" s="17" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H23" s="15" t="inlineStr">
+      <c r="H23" s="13" t="inlineStr">
         <is>
           <t>DATA-02</t>
         </is>
       </c>
-      <c r="I23" s="15" t="inlineStr">
+      <c r="I23" s="13" t="inlineStr">
         <is>
           <t>Fast-selling, profitable models rank highest in the restock recommendations.</t>
         </is>
       </c>
-      <c r="J23" s="15" t="inlineStr">
+      <c r="J23" s="13" t="inlineStr">
         <is>
           <t>Distinct from Deal Radar buy ALERTS (live market offers). This is own-history restock guidance.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="91" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
+    <row r="24" ht="91" customHeight="1" s="27">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>BUY-02</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Buy Signals &amp; Funding</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall provide a funding-scenario tool: given a budget, it spreads that budget across the top restock candidates (filling the budget greedily), shows the projected cost and profit, and lets the user exclude individual models — which frees their budget for the next candidates — with the ability to restore them.</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E24" s="18" t="inlineStr">
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H24" s="11" t="inlineStr">
+      <c r="H24" s="9" t="inlineStr">
         <is>
           <t>BUY-01</t>
         </is>
       </c>
-      <c r="I24" s="11" t="inlineStr">
+      <c r="I24" s="9" t="inlineStr">
         <is>
           <t>A budget produces a ranked, affordable shopping list; excluding an item frees its budget and pulls in the next pick.</t>
         </is>
       </c>
-      <c r="J24" s="11" t="inlineStr">
+      <c r="J24" s="9" t="inlineStr">
         <is>
           <t>Excluding a model frees its budget; the allocation pulls in the next pick.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="52" customHeight="1">
-      <c r="A25" s="14" t="inlineStr">
+    <row r="25" ht="52" customHeight="1" s="27">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>BUY-03</t>
         </is>
       </c>
-      <c r="B25" s="15" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>Buy Signals &amp; Funding</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall provide a 'watches to sell' list that highlights which items to move first — worst inventory grade first, then the items with the most capital tied up.</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E25" s="16" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F25" s="17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G25" s="17" t="inlineStr">
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H25" s="15" t="inlineStr">
+      <c r="H25" s="13" t="inlineStr">
         <is>
           <t>INV-03</t>
         </is>
       </c>
-      <c r="I25" s="15" t="inlineStr">
+      <c r="I25" s="13" t="inlineStr">
         <is>
           <t>Aged, high-cost stock appears at the top of the list.</t>
         </is>
       </c>
-      <c r="J25" s="15" t="inlineStr">
+      <c r="J25" s="13" t="inlineStr">
         <is>
           <t>Validated in POC.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="52" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
+    <row r="26" ht="52" customHeight="1" s="27">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>PROJ-01</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Projections</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall show projected profit — the target wholesale price minus cost — summed across the inventory that has a target price set.</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E26" s="18" t="inlineStr">
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F26" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G26" s="13" t="inlineStr">
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H26" s="11" t="inlineStr">
+      <c r="H26" s="9" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="I26" s="11" t="inlineStr">
+      <c r="I26" s="9" t="inlineStr">
         <is>
           <t>Projected profit sums correctly over the items that have a target price.</t>
         </is>
       </c>
-      <c r="J26" s="11" t="inlineStr">
+      <c r="J26" s="9" t="inlineStr">
         <is>
           <t>Only the target-priced portion counts.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="65" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
+    <row r="27" ht="65" customHeight="1" s="27">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>PROJ-02</t>
         </is>
       </c>
-      <c r="B27" s="15" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Projections</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall compare projected profit against historically realized profit, by model and by brand, so the user can see whether projected margins line up with what the business has actually achieved.</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E27" s="19" t="inlineStr">
+      <c r="E27" s="17" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F27" s="17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G27" s="17" t="inlineStr">
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H27" s="15" t="inlineStr">
+      <c r="H27" s="13" t="inlineStr">
         <is>
           <t>DATA-01,DATA-02</t>
         </is>
       </c>
-      <c r="I27" s="15" t="inlineStr">
+      <c r="I27" s="13" t="inlineStr">
         <is>
           <t>Each model and brand shows its projected margin alongside its historically realized margin.</t>
         </is>
       </c>
-      <c r="J27" s="15" t="inlineStr">
+      <c r="J27" s="13" t="inlineStr">
         <is>
           <t>Validated in POC.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="52" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
+    <row r="28" ht="52" customHeight="1" s="27">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>LIAB-01</t>
         </is>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Liabilities</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall show the unpaid-inventory liability — the total the business still owes on inventory it has not yet paid for.</t>
         </is>
       </c>
-      <c r="D28" s="11" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F28" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H28" s="11" t="inlineStr">
+      <c r="H28" s="9" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="I28" s="11" t="inlineStr">
+      <c r="I28" s="9" t="inlineStr">
         <is>
           <t>The unpaid total matches the outstanding balances of the unpaid items.</t>
         </is>
       </c>
-      <c r="J28" s="11" t="inlineStr">
+      <c r="J28" s="9" t="inlineStr">
         <is>
           <t>Reflects full dataset; ignores brand/period filters.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="52" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
+    <row r="29" ht="52" customHeight="1" s="27">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>LIAB-02</t>
         </is>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Liabilities</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall show consignment and memo liability — the value of goods the business holds on consignment or on memo, which it does not own outright.</t>
         </is>
       </c>
-      <c r="D29" s="15" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E29" s="16" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F29" s="17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G29" s="17" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H29" s="15" t="inlineStr">
+      <c r="H29" s="13" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="I29" s="15" t="inlineStr">
+      <c r="I29" s="13" t="inlineStr">
         <is>
           <t>The consignment and memo total matches those items.</t>
         </is>
       </c>
-      <c r="J29" s="15" t="inlineStr"/>
-    </row>
-    <row r="30" ht="46" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="J29" s="13" t="n"/>
+    </row>
+    <row r="30" ht="46" customHeight="1" s="27">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>LIAB-03</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Liabilities</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall list overpaid invoices — invoices with a negative balance, where more was paid than was owed.</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E30" s="18" t="inlineStr">
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F30" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="inlineStr">
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H30" s="11" t="inlineStr">
+      <c r="H30" s="9" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="I30" s="11" t="inlineStr">
+      <c r="I30" s="9" t="inlineStr">
         <is>
           <t>Invoices with a negative balance are listed and totalled.</t>
         </is>
       </c>
-      <c r="J30" s="11" t="inlineStr"/>
-    </row>
-    <row r="31" ht="46" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="J30" s="9" t="n"/>
+    </row>
+    <row r="31" ht="46" customHeight="1" s="27">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>LIAB-04</t>
         </is>
       </c>
-      <c r="B31" s="15" t="inlineStr">
+      <c r="B31" s="13" t="inlineStr">
         <is>
           <t>Liabilities</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="C31" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall show an estimate of sales tax owed, grouped by state.</t>
         </is>
       </c>
-      <c r="D31" s="15" t="inlineStr">
+      <c r="D31" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E31" s="19" t="inlineStr">
+      <c r="E31" s="17" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F31" s="17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G31" s="17" t="inlineStr">
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G31" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H31" s="15" t="inlineStr">
+      <c r="H31" s="13" t="inlineStr">
         <is>
           <t>DATA-02</t>
         </is>
       </c>
-      <c r="I31" s="15" t="inlineStr">
+      <c r="I31" s="13" t="inlineStr">
         <is>
           <t>The sales-tax estimate is grouped by state.</t>
         </is>
       </c>
-      <c r="J31" s="15" t="inlineStr">
+      <c r="J31" s="13" t="inlineStr">
         <is>
           <t>Validated in POC.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="78" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
+    <row r="32" ht="78" customHeight="1" s="27">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>GRADE-01</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>Grading &amp; Config</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>The per-sale performance grade shall be tunable per business: a user in the admin tier can adjust how much margin versus selling speed counts, the thresholds for each, and the overall harshness. The chosen settings apply to everyone in the business.</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="D32" s="9" t="inlineStr">
         <is>
           <t>Admin tier</t>
         </is>
       </c>
-      <c r="E32" s="18" t="inlineStr">
+      <c r="E32" s="16" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F32" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G32" s="13" t="inlineStr">
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H32" s="11" t="inlineStr">
+      <c r="H32" s="9" t="inlineStr">
         <is>
           <t>SALES-03,PLAT-04</t>
         </is>
       </c>
-      <c r="I32" s="11" t="inlineStr">
+      <c r="I32" s="9" t="inlineStr">
         <is>
           <t>Changing the weighting re-grades all of that business's sales consistently.</t>
         </is>
       </c>
-      <c r="J32" s="11" t="inlineStr">
+      <c r="J32" s="9" t="inlineStr">
         <is>
           <t>Formula in Impl. Notes.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="52" customHeight="1">
-      <c r="A33" s="14" t="inlineStr">
+    <row r="33" ht="52" customHeight="1" s="27">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>GRADE-02</t>
         </is>
       </c>
-      <c r="B33" s="15" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Grading &amp; Config</t>
         </is>
       </c>
-      <c r="C33" s="15" t="inlineStr">
+      <c r="C33" s="13" t="inlineStr">
         <is>
           <t>The inventory aging grade shall be tunable per business: a user in the admin tier can set the day thresholds that map to grades A through F.</t>
         </is>
       </c>
-      <c r="D33" s="15" t="inlineStr">
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>Admin tier</t>
         </is>
       </c>
-      <c r="E33" s="19" t="inlineStr">
+      <c r="E33" s="17" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F33" s="17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G33" s="17" t="inlineStr">
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H33" s="15" t="inlineStr">
+      <c r="H33" s="13" t="inlineStr">
         <is>
           <t>INV-03</t>
         </is>
       </c>
-      <c r="I33" s="15" t="inlineStr">
+      <c r="I33" s="13" t="inlineStr">
         <is>
           <t>Changing the day thresholds re-buckets the inventory into new grades.</t>
         </is>
       </c>
-      <c r="J33" s="15" t="inlineStr"/>
-    </row>
-    <row r="34" ht="52" customHeight="1">
-      <c r="A34" s="10" t="inlineStr">
+      <c r="J33" s="13" t="n"/>
+    </row>
+    <row r="34" ht="52" customHeight="1" s="27">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>UI-01</t>
         </is>
       </c>
-      <c r="B34" s="11" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Detail &amp; UI</t>
         </is>
       </c>
-      <c r="C34" s="11" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall present four tabs — Inventory, Sales, Buy Signals, and Liabilities. Live dealer-message alerts are handled by the separate Deal Radar feature, not here.</t>
         </is>
       </c>
-      <c r="D34" s="11" t="inlineStr">
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F34" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G34" s="13" t="inlineStr">
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H34" s="11" t="inlineStr"/>
-      <c r="I34" s="11" t="inlineStr">
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="inlineStr">
         <is>
           <t>The four tabs each render their respective analytics.</t>
         </is>
       </c>
-      <c r="J34" s="11" t="inlineStr"/>
-    </row>
-    <row r="35" ht="65" customHeight="1">
-      <c r="A35" s="14" t="inlineStr">
+      <c r="J34" s="9" t="n"/>
+    </row>
+    <row r="35" ht="65" customHeight="1" s="27">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>UI-02</t>
         </is>
       </c>
-      <c r="B35" s="15" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Detail &amp; UI</t>
         </is>
       </c>
-      <c r="C35" s="15" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>Global filters — brand, status, and time period — shall apply across the analytic views. The Liabilities view is a deliberate exception: it always shows full financial exposure and ignores these filters.</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E35" s="19" t="inlineStr">
+      <c r="E35" s="17" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F35" s="17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G35" s="17" t="inlineStr">
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H35" s="15" t="inlineStr"/>
-      <c r="I35" s="15" t="inlineStr">
+      <c r="H35" s="13" t="n"/>
+      <c r="I35" s="13" t="inlineStr">
         <is>
           <t>Applying a brand filter narrows the analytic views but not the liabilities figures.</t>
         </is>
       </c>
-      <c r="J35" s="15" t="inlineStr">
+      <c r="J35" s="13" t="inlineStr">
         <is>
           <t>Liabilities = real financial exposure, always full.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="65" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
+    <row r="36" ht="65" customHeight="1" s="27">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>UI-03</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Detail &amp; UI</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>The dashboard shall support click-through drill-down throughout — for example from a brand to its models, from a salesperson to their sales, and from a model to its individual items.</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E36" s="18" t="inlineStr">
+      <c r="E36" s="16" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G36" s="13" t="inlineStr">
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H36" s="11" t="inlineStr"/>
-      <c r="I36" s="11" t="inlineStr">
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="inlineStr">
         <is>
           <t>Clicking a summary row reveals the detail behind it.</t>
         </is>
       </c>
-      <c r="J36" s="11" t="inlineStr"/>
-    </row>
-    <row r="37" ht="78" customHeight="1">
-      <c r="A37" s="14" t="inlineStr">
+      <c r="J36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="78" customHeight="1" s="27">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>UI-04</t>
         </is>
       </c>
-      <c r="B37" s="15" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>Detail &amp; UI</t>
         </is>
       </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="C37" s="13" t="inlineStr">
         <is>
           <t>Within an analysis such as the funding scenarios, a user shall be able to exclude or adjust items and later restore them; the change affects that analysis view. Ad-hoc view tweaks are personal to the user, while saved business-wide configuration is admin-tier.</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
+      <c r="D37" s="13" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E37" s="19" t="inlineStr">
+      <c r="E37" s="17" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F37" s="17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G37" s="17" t="inlineStr">
+      <c r="F37" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H37" s="15" t="inlineStr">
+      <c r="H37" s="13" t="inlineStr">
         <is>
           <t>BUY-02</t>
         </is>
       </c>
-      <c r="I37" s="15" t="inlineStr">
+      <c r="I37" s="13" t="inlineStr">
         <is>
           <t>Excluding an item updates the analysis and can be undone.</t>
         </is>
       </c>
-      <c r="J37" s="15" t="inlineStr">
+      <c r="J37" s="13" t="inlineStr">
         <is>
           <t>Saved/shared config is admin-tier; ad-hoc view tweaks are per-user.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="52" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
+    <row r="38" ht="52" customHeight="1" s="27">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>NFR-01</t>
         </is>
       </c>
-      <c r="B38" s="11" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>Non-Functional</t>
         </is>
       </c>
-      <c r="C38" s="11" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>The system shall keep each business's inventory, sales, configuration, and all derived analytics strictly isolated from every other business.</t>
         </is>
       </c>
-      <c r="D38" s="11" t="inlineStr">
+      <c r="D38" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F38" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G38" s="13" t="inlineStr">
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="H38" s="11" t="inlineStr">
+      <c r="H38" s="9" t="inlineStr">
         <is>
           <t>PLAT-04</t>
         </is>
       </c>
-      <c r="I38" s="11" t="inlineStr">
+      <c r="I38" s="9" t="inlineStr">
         <is>
           <t>No path allows one business to read another business's data.</t>
         </is>
       </c>
-      <c r="J38" s="11" t="inlineStr"/>
-    </row>
-    <row r="39" ht="65" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
+      <c r="J38" s="9" t="n"/>
+    </row>
+    <row r="39" ht="65" customHeight="1" s="27">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>NFR-02</t>
         </is>
       </c>
-      <c r="B39" s="15" t="inlineStr">
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>Non-Functional</t>
         </is>
       </c>
-      <c r="C39" s="15" t="inlineStr">
+      <c r="C39" s="13" t="inlineStr">
         <is>
           <t>The dashboard shall compute its analytics across a business's full inventory and sales history within a responsive time budget, using caching or incremental computation where needed.</t>
         </is>
       </c>
-      <c r="D39" s="15" t="inlineStr">
+      <c r="D39" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E39" s="19" t="inlineStr">
+      <c r="E39" s="17" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F39" s="17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G39" s="17" t="inlineStr">
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H39" s="15" t="inlineStr"/>
-      <c r="I39" s="15" t="inlineStr">
+      <c r="H39" s="13" t="n"/>
+      <c r="I39" s="13" t="inlineStr">
         <is>
           <t>The dashboard loads and recomputes within an acceptable time on a full dataset.</t>
         </is>
       </c>
-      <c r="J39" s="15" t="inlineStr">
+      <c r="J39" s="13" t="inlineStr">
         <is>
           <t>POC caches the WatchOps pulls.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="65" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
+    <row r="40" ht="65" customHeight="1" s="27">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>NFR-03</t>
         </is>
       </c>
-      <c r="B40" s="11" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>Non-Functional</t>
         </is>
       </c>
-      <c r="C40" s="11" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>When reading inventory from WatchOps, the system shall page through all records, exclude items that are sold or voided, and correctly map the inventory types (owned, memo, partnership, consignment).</t>
         </is>
       </c>
-      <c r="D40" s="11" t="inlineStr">
+      <c r="D40" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E40" s="10" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F40" s="13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G40" s="13" t="inlineStr">
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="H40" s="11" t="inlineStr">
+      <c r="H40" s="9" t="inlineStr">
         <is>
           <t>DATA-01</t>
         </is>
       </c>
-      <c r="I40" s="11" t="inlineStr">
+      <c r="I40" s="9" t="inlineStr">
         <is>
           <t>All live holdings load, sold and voided items are excluded, and inventory types are correctly assigned.</t>
         </is>
       </c>
-      <c r="J40" s="11" t="inlineStr">
+      <c r="J40" s="9" t="inlineStr">
         <is>
           <t>Validated in POC.</t>
         </is>
@@ -2881,192 +2872,188 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" style="27" min="1" max="1"/>
+    <col width="17" customWidth="1" style="27" min="2" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+    <row r="1" ht="20" customHeight="1" s="27">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>Roles &amp; Permissions</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Everyone views everything; roles gate CONFIGURATION only. ✓ = allowed.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+    <row r="4" ht="42" customHeight="1" s="27">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Capability</t>
         </is>
       </c>
-      <c r="B4" s="22" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Administrator</t>
         </is>
       </c>
-      <c r="C4" s="22" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>Sales Personnel Admin</t>
         </is>
       </c>
-      <c r="D4" s="22" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>Sales Personnel Viewer</t>
         </is>
       </c>
-      <c r="E4" s="22" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>Back Office Viewer</t>
         </is>
       </c>
-      <c r="F4" s="22" t="inlineStr">
+      <c r="F4" s="20" t="inlineStr">
         <is>
           <t>Data Entry Assistant</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="23" t="inlineStr">
+    <row r="5" ht="30" customHeight="1" s="27">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>View all analytics (incl. cost, margin, liabilities, all staff)</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="D5" s="24" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E5" s="24" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F5" s="24" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
+    <row r="6" ht="30" customHeight="1" s="27">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Adjust filters / exclusions (own view)</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C6" s="24" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="F6" s="24" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="23" t="inlineStr">
+    <row r="7" ht="30" customHeight="1" s="27">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Configure grading formula (business-wide)</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="D7" s="25" t="inlineStr"/>
-      <c r="E7" s="25" t="inlineStr"/>
-      <c r="F7" s="25" t="inlineStr"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="D7" s="23" t="n"/>
+      <c r="E7" s="23" t="n"/>
+      <c r="F7" s="23" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1" s="27">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Manage data sources &amp; settings</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="C8" s="25" t="inlineStr"/>
-      <c r="D8" s="25" t="inlineStr"/>
-      <c r="E8" s="25" t="inlineStr"/>
-      <c r="F8" s="25" t="inlineStr"/>
+      <c r="C8" s="23" t="n"/>
+      <c r="D8" s="23" t="n"/>
+      <c r="E8" s="23" t="n"/>
+      <c r="F8" s="23" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="26" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>• Admin tier = Administrator + Sales Personnel Admin (both configure the grading formula).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>• Manage data sources &amp; settings (connecting WatchOps, defaults) is Administrator-only by default — extendable in one cell.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>• 'Everyone views everything' is a deliberate decision: no role hides cost, margin, liabilities, or another salesperson's numbers.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>• Ad-hoc view tweaks (filters, per-view exclusions) are personal and non-destructive; saved business-wide config is admin-tier.</t>
         </is>
@@ -3090,118 +3077,118 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:C12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="94" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" style="27" min="1" max="1"/>
+    <col width="30" customWidth="1" style="27" min="2" max="2"/>
+    <col width="94" customWidth="1" style="27" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="20" t="inlineStr">
+    <row r="2" ht="20" customHeight="1" s="27">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Implementation Notes — formulas &amp; lessons from the POC</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="B3" s="28" t="inlineStr">
+    <row r="3" ht="30" customHeight="1" s="27">
+      <c r="B3" s="30" t="inlineStr">
         <is>
           <t>The fresh build reuses no POC code but should reproduce these exactly. Each was worked out against the live WatchOps API and real dealer data.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="72" customHeight="1">
-      <c r="B5" s="29" t="inlineStr">
+    <row r="5" ht="72" customHeight="1" s="27">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>WatchOps API returns numeric codes; the export shows text</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Derived by joining a real export to the API on INVENTORY ID (2,146/2,146 rows agreed). CONDITION: 4=New, 3=Retail Ready/Like New, 2=Mint/Very Good, 1 and 10=Used/Good. INVENTORY_STATUS: 1=Inhand, 2=Incoming, 3=Out on Memo, 4=On Hold/Reserved, 6=Needs Service/Polish, 7=At Service, 10=Sold &amp; Cashed Out. Box/papers: warrantybox / warrantypaper = '1' means yes. The older watchbi-app had the CONDITION map INVERTED — do not copy it; use this.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="96" customHeight="1">
-      <c r="B6" s="29" t="inlineStr">
+    <row r="6" ht="96" customHeight="1" s="27">
+      <c r="B6" s="25" t="inlineStr">
         <is>
           <t>DJ sales grade (per-sale performance)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Points system, 'each data point is 1 point' (DJ Allen). Two factors: Margin (GP% = profit/cost) and Velocity (days on hand). Each factor → points A=4/B=3/C=2/D=1 by thresholds (default margin GP%: A&gt;=30, B&gt;=20, C&gt;=10). Weighted score = (marginPts*Wmargin + daysPts*Wvelocity) / (Wmargin+Wvelocity), with marginWeight default 50 (velocity weight = 100-marginWeight). Grade: A if score&gt;=3.5+shift, B&gt;=2.5+shift, C&gt;=1.5+shift, else D, where 'shift' is a harshness lever. Weights, thresholds, and harshness are per-business configurable. Uses NO market data.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="B7" s="29" t="inlineStr">
+    <row r="7" ht="36" customHeight="1" s="27">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>Inventory quality grade (A→F) and aging</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Grade by days in stock: A = fresh, F = aged (thresholds configurable). 'Watches to sell' ranks worst grade first, then most capital tied up. 91+ days is the headline 'aged' KPI.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="B8" s="29" t="inlineStr">
+    <row r="8" ht="60" customHeight="1" s="27">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>Velocity / weeks-of-stock</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>weeklyVelocity from recent (windowed) unit sales; weeksOfStock = stock / weeklyVelocity. Guard sparse/single-sale windows so they don't overstate velocity (a lone recent sale shouldn't imply infinite demand). Some references are deliberately excluded from velocity/median math — keep the unit counted but drop its days-to-sell.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="B9" s="29" t="inlineStr">
+    <row r="9" ht="48" customHeight="1" s="27">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>Projected profit</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Projected profit = target wholesale price − cost, computed only over the priced (target-bearing) portion of inventory. Projected-vs-historical compares this to the margin the same model/brand actually realized in sales.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="B10" s="29" t="inlineStr">
+    <row r="10" ht="48" customHeight="1" s="27">
+      <c r="B10" s="25" t="inlineStr">
         <is>
           <t>Liabilities are full-exposure</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Unpaid inventory, consignment/memo, overpaid invoices, and sales tax reflect real financial exposure across the ENTIRE dataset and intentionally ignore the brand/status/period filters. Compute them independently of the filtered analytic views.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="B11" s="29" t="inlineStr">
+    <row r="11" ht="60" customHeight="1" s="27">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>Inventory ingestion details</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>WatchOps inventory is paginated (POST /inventories, ~250/page). Exclude sold and voided items (status contains 'void', or voidreason set). Inventory type maps owned / memo / partnership / consignment. Filter fully-blank rows (no brand AND no model) at the source so they don't pollute any total.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="B12" s="29" t="inlineStr">
+    <row r="12" ht="60" customHeight="1" s="27">
+      <c r="B12" s="25" t="inlineStr">
         <is>
           <t>WatchCharts is removed</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>The POC compared cost/target/sale price to WatchCharts market value (median asking, dealer price, market price) — Oldest-20 and Latest-20 'market grade' views, and a market-based sales grade. All of that is OUT for v1. The DJ sales grade (margin+velocity) and everything else are built on the business's own data and remain.</t>
         </is>
@@ -3222,87 +3209,87 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:C14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="92" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" style="27" min="1" max="1"/>
+    <col width="30" customWidth="1" style="27" min="2" max="2"/>
+    <col width="92" customWidth="1" style="27" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="20" t="inlineStr">
+    <row r="2" ht="20" customHeight="1" s="27">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Backlog &amp; Open Items</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Billing granularity</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Per-business vs per-seat unlock — deferred; affects only the entitlement check (PLAT-01).</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="8" t="inlineStr">
+    <row r="6" ht="28" customHeight="1" s="27">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Market data (if WatchOps adds it)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>WatchCharts is removed. If WatchOps later exposes market/pricing data, the market-comparison views (stock vs market, market-based sale grade) could return — spec them then.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Sales trends over time</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>A time-series sales view existed in an earlier POC and was removed. Reconsider if wanted.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="8" t="inlineStr">
+    <row r="10" ht="28" customHeight="1" s="27">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Non-WatchOps businesses</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Excel/CSV upload (DATA-05) already lets a non-WatchOps business use the dashboard. A live Google-Sheet/API connector (auto-refreshing, vs a one-off upload) is the remaining open question.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Grading defaults</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Confirm the default DJ-grade thresholds and aging-day cutoffs to ship before a business tunes them.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Export / reporting</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Whether views need CSV/PDF export or scheduled reports — not in the current POC.</t>
         </is>

</xml_diff>

<commit_message>
Move fast-follow (Should) requirements to Phase 2; Must stays Phase 1
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WatchBI_Dashboard_Requirements.xlsx
+++ b/WatchBI_Dashboard_Requirements.xlsx
@@ -1627,7 +1627,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G26" s="11" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="F27" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G27" s="15" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="F31" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G31" s="15" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="F33" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="F35" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G35" s="15" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G36" s="11" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="F37" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G37" s="15" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="F39" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G39" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Fix WatchCharts market grades to compare prices at matching levels
Grade each of our prices against the WatchCharts value at the same
market level: retail target (tag / end-customer) vs median asking,
wholesale target vs dealer price, cost vs dealer price (market_price
fallback). Adds the QoW wholesale check and wires up the previously
unused dealerPrice / market_price fields. Also add targetEndCustomer
to the inventory mapping. Includes updated requirement docs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WatchBI_Dashboard_Requirements.xlsx
+++ b/WatchBI_Dashboard_Requirements.xlsx
@@ -998,7 +998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col hidden="1" width="11" customWidth="1" style="33" min="1" max="1"/>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C3" s="17" t="inlineStr">
         <is>
-          <t>The dashboard shall run as its own website on a subdomain of WatchOps (for example watchbi.watchops.com) — a sibling to Deal Radar, which lives on its own subdomain under the same WatchOps domain.</t>
+          <t>The dashboard shall run as its own website on a subdomain of WatchOps (for example watchbi.watchops.com) — a sibling to Deal Radar. It shall be reachable from WatchOps' top-right admin menu, and shown with a lock icon for accounts that do not have the subscription.</t>
         </is>
       </c>
       <c r="D3" s="17" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>The dashboard shall provide a supplier view showing spend, unit count, and aging grouped by supplier (top suppliers).</t>
+          <t>The dashboard shall provide a supplier view showing spend, unit count, aging, and gross profit grouped by supplier (top suppliers).</t>
         </is>
       </c>
       <c r="D19" s="17" t="inlineStr">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
-          <t>Supplier totals reconcile with the inventory.</t>
+          <t>Supplier totals, including gross profit, reconcile with the inventory.</t>
         </is>
       </c>
       <c r="H19" s="17" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>Exact formula in Impl. Notes. Does NOT use market data.</t>
+          <t>Exact formula in Impl. Notes. Does NOT use market data. Grading formula still to be decided.</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>Reflects full dataset; ignores brand/period filters.</t>
+          <t>Reflects full dataset; ignores filters. Depends on WatchOps tracking paid/unpaid, which WYW does not use yet (Trello today); usable once that is in place.</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,11 @@
           <t>Invoices with a negative balance are listed and totalled.</t>
         </is>
       </c>
-      <c r="H33" s="17" t="n"/>
+      <c r="H33" s="17" t="inlineStr">
+        <is>
+          <t>Sourced from the WatchOps invoice section.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="46" customHeight="1" s="33">
       <c r="A34" s="12" t="inlineStr">
@@ -2874,7 +2878,7 @@
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>The dashboard shall compute every sales metric in two mutually exclusive bases. CLOSED = a sale booked/marked sold but not yet cashed out (a WatchOps status such as 'Shipped waiting on payment' or 'Invoiced'). CASHED = the WatchOps status 'Sold &amp; Cashed Out', which a business reaches only once the item is fully paid, has a tracking number, and has passed through 'Shipped waiting on payment'. A deal counts as Closed until it becomes Cashed — never both.</t>
+          <t>The dashboard shall compute every sales metric in two mutually exclusive bases. CLOSED = a sale booked/marked sold but not yet cashed out (a WatchOps status such as 'Shipped waiting on payment', 'Need to Ship', or 'Invoiced'). CASHED = the WatchOps status 'Sold &amp; Cashed Out', which a business reaches only once the item is fully paid, has a tracking number, and has passed through 'Shipped waiting on payment'. The closed-to-cashed change and the lock/unlock happen in WatchOps (by role); God's Eye reflects them automatically, with no manual step in the dashboard. A deal counts as Closed until it becomes Cashed — never both. MONTH ATTRIBUTION: a deal is counted in the Closed basis in the month it closed, and in the Cashed basis in the month it becomes fully cashed — which may be a later month.</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
@@ -2899,7 +2903,7 @@
       </c>
       <c r="H46" s="13" t="inlineStr">
         <is>
-          <t>Status meanings in Impl. Notes. The cashing gate lives in WatchOps, not this dashboard.</t>
+          <t>Status meanings in Impl. Notes. Cash/lock lives in WatchOps and reflects automatically. Closed and Cashed for the same deal can fall in different months.</t>
         </is>
       </c>
     </row>
@@ -2958,7 +2962,7 @@
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>For each salesperson and month, the God's Eye table shall show a GP Budget and a Unit Budget (from the Salesperson Budget tab, SCORE-01), plus Pacing and Over/Under for GP, Units, and Revenue in both bases. Pacing is a value the manager ENTERS (their projection of where the month lands), not a figure the system extrapolates. Over/Under = pacing minus budget.</t>
+          <t>For each salesperson and month, the God's Eye table shall show a GP Budget and a Unit Budget (entered by managers, from the Salesperson Budget tab, SCORE-01). The dashboard shall CALCULATE Pacing and Over/Under for GP and Units automatically from calendar days elapsed (days passed vs. days in the month) against actuals — managers enter budgets only, never pacing or over/under. Revenue shows an actual and a Pacing figure but no budget and no Over/Under.</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
@@ -2978,12 +2982,12 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>Budget, manager-entered pacing, and over/under show for GP, Units, and Revenue in both Closed and Cashed bases.</t>
+          <t>Managers enter budgets; the dashboard computes pacing and over/under for GP and Units from calendar days. Revenue shows actual and pacing only, in both bases.</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
-          <t>Pacing is manager-set per decision. Budgets come from SCORE-01.</t>
+          <t>CHANGED per 2026-08-21 meeting: pacing/over-under are dashboard-calculated from calendar days, not manager-entered. Budgets come from SCORE-01.</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3046,7 @@
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>The admin tier shall set, each month, a team-wide sales goal for the whole sales team — a total GP goal and a total units goal — entered roughly a week before the month begins.</t>
+          <t>Managers (admin tier) shall set monthly budgets both company-wide and per salesperson — a GP goal and a units goal at each level — entered roughly a week before the month begins.</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
@@ -3062,12 +3066,12 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>An owner/manager can enter a team GP goal and units goal for a given month.</t>
+          <t>An owner/manager can enter company-wide and per-salesperson GP and units budgets for a given month.</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
-          <t>Feeds the God's Eye budget columns (SALES-08).</t>
+          <t>Feeds the God's Eye budget columns (SALES-08). Per-salesperson AND company-wide, per 2026-08-21 meeting.</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3088,7 @@
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>The team goal shall be split into a per-salesperson budget automatically, in proportion to each salesperson's share of sales over the trailing three months, with the admin tier able to override any individual's number by hand.</t>
+          <t>Per-salesperson budgets may be seeded automatically from each salesperson's share of sales over the trailing three months, and then edited by hand.</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
@@ -3104,7 +3108,7 @@
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>The team goal divides across salespeople by their trailing-3-month share; an admin can override any figure.</t>
+          <t>The system can propose per-salesperson budgets from trailing-3-month share; an admin can override any figure.</t>
         </is>
       </c>
       <c r="H51" s="13" t="inlineStr">
@@ -3126,7 +3130,7 @@
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>The dashboard shall provide a Sales Scoreboard that tracks, each month, each salesperson's attainment against their budget — revenue and units, actual vs goal, with over/under.</t>
+          <t>The dashboard shall provide a Sales Scoreboard that tracks, each month, each salesperson's attainment against budget — revenue and units, actual vs goal, with over/under calculated from calendar days elapsed.</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
@@ -3206,7 +3210,7 @@
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>The funding-scenario tool shall accept a target days-of-stock (day-supply) level. It shall first allocate the budget to reach that day-supply across the restock candidates; any budget remaining after the target is met shall be shown separately as surplus, with suggested additional buys for it. Example: a $500k budget with a 90-day target that needs only $250k of stock shows the $250k that reaches 90 days, then the $250k of surplus to deploy.</t>
+          <t>The funding-scenario tool shall accept a dual input of budget (money) and target days-of-stock (time), with both recommended and manual entry. It shall show which watches to buy to reach the target, and how that spend changes budget forecasting going forward (e.g. $400k deployed over 40 days).</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
@@ -3226,12 +3230,12 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>Given a budget and a days-of-stock target, the tool shows the buys that reach the target and, separately, the leftover budget with suggestions.</t>
+          <t>Given a budget and/or a days-of-stock target, the tool recommends buys, accepts manual adjustment, and shows the forward budget/forecasting impact.</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr">
         <is>
-          <t>Extends BUY-02. Day-supply derived from velocity / weeks-of-stock (INV-04).</t>
+          <t>Extends BUY-02. Dual money+time input and forecasting impact per 2026-08-21 meeting.</t>
         </is>
       </c>
     </row>
@@ -3316,6 +3320,86 @@
       <c r="H56" s="13" t="inlineStr">
         <is>
           <t>Complements INV-05, which is current-inventory spend and aging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>SALES-10</t>
+        </is>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>Sales Analytics</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>Salespeople shall appear or disappear from the God's Eye view by calendar month automatically, based on their WatchOps activation and deactivation dates — shown in the months they were active, hidden in the months they were not — so reports never need manual reconfiguration when staff are hired or let go.</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F57" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="13" t="inlineStr">
+        <is>
+          <t>A salesperson shows only in the months they were active per their WatchOps activation/deactivation dates; no manual reconfiguration is needed.</t>
+        </is>
+      </c>
+      <c r="H57" s="13" t="inlineStr">
+        <is>
+          <t>Top client pain point (2026-08-21): today the God's Eye report is rebuilt by hand for a week whenever staff change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>LIAB-05</t>
+        </is>
+      </c>
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>Liabilities</t>
+        </is>
+      </c>
+      <c r="C58" s="13" t="inlineStr">
+        <is>
+          <t>The dashboard shall provide a sales-tax dashboard showing tax collected per state, and how much of it has been paid versus still owed (invoiced is not the same as paid).</t>
+        </is>
+      </c>
+      <c r="D58" s="13" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E58" s="22" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="F58" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G58" s="13" t="inlineStr">
+        <is>
+          <t>Sales tax is shown per state as collected, paid, and still owed.</t>
+        </is>
+      </c>
+      <c r="H58" s="13" t="inlineStr">
+        <is>
+          <t>Future / later phase (2026-08-21). Extends LIAB-04 beyond a single owed total.</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3436,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="33">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -3506,7 +3589,6 @@
       <c r="D10" s="29" t="n"/>
       <c r="E10" s="29" t="n"/>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="30" t="inlineStr">
         <is>
@@ -3679,6 +3761,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="64" customHeight="1" s="33">
       <c r="B14" s="31" t="inlineStr">
         <is>
@@ -3692,7 +3775,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" s="31" t="inlineStr">
         <is>
           <t>God's Eye columns (per salesperson, per month)</t>
@@ -3700,12 +3782,11 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>One row per Sales Associate (WatchOps 'sold by'), plus Average and Total rows. Columns, in order: Sales Associate; Closed GP; Cashed GP; GP Budget; Pacing GP Closed; Pacing GP Cashed; Over/Under GP Closed; Over/Under GP Cashed; Units Closed; Units Cashed; Unit Budget; Pacing Units Closed; Pacing Units Cashed; Over/Under Units Closed; Over/Under Units Cashed; Revenue Closed; Revenue Cashed; Pacing Revenue Closed; Pacing Revenue Cashed; GP/PU Closed; GP/PU Cashed; Average Aging Closed; Average Aging Cashed; Margin Closed; Margin Cashed; Average Price Closed; Average Price Cashed. Pacing columns are MANAGER-ENTERED projections, not system-extrapolated. Over/Under = pacing - budget.</t>
+          <t>One row per Sales Associate (WatchOps 'sold by'), plus Average and Total rows. Columns, in order: Sales Associate; Closed GP; Cashed GP; GP Budget; Pacing GP Closed; Pacing GP Cashed; Over/Under GP Closed; Over/Under GP Cashed; Units Closed; Units Cashed; Unit Budget; Pacing Units Closed; Pacing Units Cashed; Over/Under Units Closed; Over/Under Units Cashed; Revenue Closed; Revenue Cashed; Pacing Revenue Closed; Pacing Revenue Cashed; GP/PU Closed; GP/PU Cashed; Average Aging Closed; Average Aging Cashed; Margin Closed; Margin Cashed; Average Price Closed; Average Price Cashed. Managers enter BUDGETS only (company-wide and per salesperson); the dashboard CALCULATES pacing and over/under for GP and Units from calendar days elapsed (changed 2026-08-21). Revenue has no budget/over-under (actual + pacing only). Salespeople show/hide by month per their WatchOps activation/deactivation dates (SALES-10).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" s="31" t="inlineStr">
         <is>
           <t>Closed vs Cashed (status mapping)</t>
@@ -3713,12 +3794,11 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>CASHED = WatchOps status 'Sold &amp; Cashed Out' (the business only lets a watch reach it once it is fully paid + has a tracking number + came through 'Shipped waiting on payment'). CLOSED = booked/marked sold but not yet cashed (e.g. 'Shipped waiting on payment', 'Invoiced', 'Need to Ship'). Mutually exclusive: a deal is Closed until it flips to Cashed. The full inventory-status dropdown seen in WatchOps includes: Inhand, Incoming, Out on Memo, On Hold/Reserved, Available to Order, Needs Service/Polish, At Service, Need to Ship, Shipped waiting on payment, Sold &amp; Cashed Out, Intake Complete, Invoiced — extend the numeric status legend to cover the ones not yet mapped (confirm codes against the API).</t>
+          <t>CASHED = WatchOps status 'Sold &amp; Cashed Out' (the business only lets a watch reach it once it is fully paid + has a tracking number + came through 'Shipped waiting on payment'). CLOSED = booked/marked sold but not yet cashed (e.g. 'Shipped waiting on payment', 'Invoiced', 'Need to Ship'). Mutually exclusive: a deal is Closed until it flips to Cashed. The full inventory-status dropdown seen in WatchOps includes: Inhand, Incoming, Out on Memo, On Hold/Reserved, Available to Order, Needs Service/Polish, At Service, Need to Ship, Shipped waiting on payment, Sold &amp; Cashed Out, Intake Complete, Invoiced — extend the numeric status legend to cover the ones not yet mapped (confirm codes against the API). MONTH: count a deal in the Cashed basis in the month it becomes fully cashed (which can be later than the month it closed); count it in the Closed basis in the month it closed.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" s="31" t="inlineStr">
         <is>
           <t>Salesperson budgets &amp; scoreboard</t>
@@ -3825,6 +3905,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -3837,8 +3918,8 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Suggested Buy dashboard (GP/Time grading)</t>

</xml_diff>